<commit_message>
Analisa os fatores condicionantes da base monetária (TCU 2010, p. 35)
Reconstrói o quadro 2003–2010 (o título cita 2002, mas a linha não foi
impressa), fecha a identidade Tesouro + títulos + externo + demais = Δ base
e documenta a troca de 2010: compulsório (−R$ 236,9 bi) no lugar das
compromissadas (+R$ 249,5 bi em títulos).

Co-authored-by: cafla19791 <cafla19791@gmail.com>
</commit_message>
<xml_diff>
--- a/output/TCU_CG_2010.xlsx
+++ b/output/TCU_CG_2010.xlsx
@@ -24,6 +24,10 @@
     <sheet name="PAC_Desoneracoes_Serie" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="PAC_Subsidios_Eixo" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Resumo_IPCA" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Base_Monetaria" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Base_Monetaria_Detalhe" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Base_Monetaria_Acum" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Base_Monetaria_IPCA" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3095,6 +3099,389 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tesouro_nacional</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>titulos_publicos</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>setor_externo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>demais_operacoes</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>var_base</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>identidade_ok</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>residuo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-1064</v>
+      </c>
+      <c r="C2" t="n">
+        <v>11181</v>
+      </c>
+      <c r="D2" t="n">
+        <v>643</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-10843</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-83</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-42140</v>
+      </c>
+      <c r="C3" t="n">
+        <v>52111</v>
+      </c>
+      <c r="D3" t="n">
+        <v>12599</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-8468</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14102</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-43008</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2808</v>
+      </c>
+      <c r="D4" t="n">
+        <v>52395</v>
+      </c>
+      <c r="E4" t="n">
+        <v>319</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12514</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-59511</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-687</v>
+      </c>
+      <c r="D5" t="n">
+        <v>74369</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5683</v>
+      </c>
+      <c r="F5" t="n">
+        <v>19854</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-55600</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-73974</v>
+      </c>
+      <c r="D6" t="n">
+        <v>155390</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-300</v>
+      </c>
+      <c r="F6" t="n">
+        <v>25516</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-74312</v>
+      </c>
+      <c r="C7" t="n">
+        <v>34059</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-12124</v>
+      </c>
+      <c r="E7" t="n">
+        <v>53311</v>
+      </c>
+      <c r="F7" t="n">
+        <v>933</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-52312</v>
+      </c>
+      <c r="C8" t="n">
+        <v>11281</v>
+      </c>
+      <c r="D8" t="n">
+        <v>62937</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-3383</v>
+      </c>
+      <c r="F8" t="n">
+        <v>18523</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-51204</v>
+      </c>
+      <c r="C9" t="n">
+        <v>249513</v>
+      </c>
+      <c r="D9" t="n">
+        <v>75553</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-233082</v>
+      </c>
+      <c r="F9" t="n">
+        <v>40780</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tesouro_nacional</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>titulos_publicos</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>setor_externo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>depositos_inst_financ</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>derivativos_ajustes</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>outras_contas_ajustes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>var_base</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>residuo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-52312</v>
+      </c>
+      <c r="C2" t="n">
+        <v>11281</v>
+      </c>
+      <c r="D2" t="n">
+        <v>62937</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-3425</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-3199</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3242</v>
+      </c>
+      <c r="H2" t="n">
+        <v>18523</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-51204</v>
+      </c>
+      <c r="C3" t="n">
+        <v>249513</v>
+      </c>
+      <c r="D3" t="n">
+        <v>75553</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-236911</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3830</v>
+      </c>
+      <c r="H3" t="n">
+        <v>40780</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4173,6 +4560,660 @@
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fator</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>acumulado_r_mi</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>acumulado_r_bi</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>anos_expansao</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>anos_retracao</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>min_r_mi</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>max_r_mi</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ano_min</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ano_max</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tesouro Nacional</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-379151</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-379.151</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-74312</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-1064</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2008</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Títulos públicos federais</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>286292</v>
+      </c>
+      <c r="C3" t="n">
+        <v>286.292</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-73974</v>
+      </c>
+      <c r="G3" t="n">
+        <v>249513</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2007</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Setor externo</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>421762</v>
+      </c>
+      <c r="C4" t="n">
+        <v>421.762</v>
+      </c>
+      <c r="D4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-12124</v>
+      </c>
+      <c r="G4" t="n">
+        <v>155390</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2008</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Demais operações</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-196763</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-196.763</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-233082</v>
+      </c>
+      <c r="G5" t="n">
+        <v>53311</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2010</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2008</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Variação da base monetária</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>132139</v>
+      </c>
+      <c r="C6" t="n">
+        <v>132.139</v>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-83</v>
+      </c>
+      <c r="G6" t="n">
+        <v>40780</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2003</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2010</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tesouro_nacional</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>titulos_publicos</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>setor_externo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>demais_operacoes</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>var_base</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>identidade_ok</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>residuo</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>fator_ipca</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>tesouro_nacional_ipca</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>titulos_publicos_ipca</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>setor_externo_ipca</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>demais_operacoes_ipca</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>var_base_ipca</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-1064</v>
+      </c>
+      <c r="C2" t="n">
+        <v>11181</v>
+      </c>
+      <c r="D2" t="n">
+        <v>643</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-10843</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-83</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.432404819188201</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-3652.078727616245</v>
+      </c>
+      <c r="K2" t="n">
+        <v>38377.71828334327</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2207.036298738013</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-37217.56545445766</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-284.8895999926207</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-42140</v>
+      </c>
+      <c r="C3" t="n">
+        <v>52111</v>
+      </c>
+      <c r="D3" t="n">
+        <v>12599</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-8468</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14102</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3.189948207730192</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-134424.4174737503</v>
+      </c>
+      <c r="K3" t="n">
+        <v>166231.391053028</v>
+      </c>
+      <c r="L3" t="n">
+        <v>40190.15746919269</v>
+      </c>
+      <c r="M3" t="n">
+        <v>-27012.48142305926</v>
+      </c>
+      <c r="N3" t="n">
+        <v>44984.64962541117</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-43008</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2808</v>
+      </c>
+      <c r="D4" t="n">
+        <v>52395</v>
+      </c>
+      <c r="E4" t="n">
+        <v>319</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12514</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.018219562813559</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-129807.5869574855</v>
+      </c>
+      <c r="K4" t="n">
+        <v>8475.160532380472</v>
+      </c>
+      <c r="L4" t="n">
+        <v>158139.6139936164</v>
+      </c>
+      <c r="M4" t="n">
+        <v>962.8120405375251</v>
+      </c>
+      <c r="N4" t="n">
+        <v>37769.99960904887</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-59511</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-687</v>
+      </c>
+      <c r="D5" t="n">
+        <v>74369</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5683</v>
+      </c>
+      <c r="F5" t="n">
+        <v>19854</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.9262823562432</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-174145.9893023891</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-2010.355978739078</v>
+      </c>
+      <c r="L5" t="n">
+        <v>217624.6925514505</v>
+      </c>
+      <c r="M5" t="n">
+        <v>16630.0626305301</v>
+      </c>
+      <c r="N5" t="n">
+        <v>58098.40990085249</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-55600</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-73974</v>
+      </c>
+      <c r="D6" t="n">
+        <v>155390</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-300</v>
+      </c>
+      <c r="F6" t="n">
+        <v>25516</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.801414074154887</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-155758.6225230117</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-207231.8047215336</v>
+      </c>
+      <c r="L6" t="n">
+        <v>435311.7329829279</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-840.4242222464661</v>
+      </c>
+      <c r="N6" t="n">
+        <v>71480.8815161361</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-74312</v>
+      </c>
+      <c r="C7" t="n">
+        <v>34059</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-12124</v>
+      </c>
+      <c r="E7" t="n">
+        <v>53311</v>
+      </c>
+      <c r="F7" t="n">
+        <v>933</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.645281282109639</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-196576.1426361315</v>
+      </c>
+      <c r="K7" t="n">
+        <v>90095.63518737219</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-32071.39026429726</v>
+      </c>
+      <c r="M7" t="n">
+        <v>141022.590430547</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2468.047436208293</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-52312</v>
+      </c>
+      <c r="C8" t="n">
+        <v>11281</v>
+      </c>
+      <c r="D8" t="n">
+        <v>62937</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-3383</v>
+      </c>
+      <c r="F8" t="n">
+        <v>18523</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.535931209916586</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-132659.6334531564</v>
+      </c>
+      <c r="K8" t="n">
+        <v>28607.839979069</v>
+      </c>
+      <c r="L8" t="n">
+        <v>159603.9025585201</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-8579.055283147809</v>
+      </c>
+      <c r="N8" t="n">
+        <v>46973.05380128491</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-51204</v>
+      </c>
+      <c r="C9" t="n">
+        <v>249513</v>
+      </c>
+      <c r="D9" t="n">
+        <v>75553</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-233082</v>
+      </c>
+      <c r="F9" t="n">
+        <v>40780</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.394441995846377</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-122605.0079553179</v>
+      </c>
+      <c r="K9" t="n">
+        <v>597444.4057096171</v>
+      </c>
+      <c r="L9" t="n">
+        <v>180907.2761121813</v>
+      </c>
+      <c r="M9" t="n">
+        <v>-558101.3292758652</v>
+      </c>
+      <c r="N9" t="n">
+        <v>97645.34459061525</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Coteja a Selic (TCU p. 33) com os fatores da base monetária (p. 35)
Cruza o desce-e-sobe da meta Copom (2003–2010) com Tesouro, títulos,
setor externo e demais operações. O gráfico da p. 33 é a janela
jan/2006–mar/2011; o cotejamento usa a série oficial SGS 432 para
casar com o quadro da p. 35.

Co-authored-by: cafla19791 <cafla19791@gmail.com>
</commit_message>
<xml_diff>
--- a/output/TCU_CG_2010.xlsx
+++ b/output/TCU_CG_2010.xlsx
@@ -27,7 +27,11 @@
     <sheet name="Base_Monetaria" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Base_Monetaria_Detalhe" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Base_Monetaria_Acum" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Base_Monetaria_IPCA" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Selic_Copom" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Selic_Anual" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Cotejamento_Selic_Base" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Selic_TCU_vs_oficial" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Base_Monetaria_IPCA" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +40,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -66,8 +73,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4788,6 +4796,1709 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>reuniao</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>vigencia</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>selic</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>delta_pp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>37608</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>37609</v>
+      </c>
+      <c r="C2" t="n">
+        <v>25</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>37643</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>37644</v>
+      </c>
+      <c r="C3" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>37671</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>37672</v>
+      </c>
+      <c r="C4" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>37790</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>37791</v>
+      </c>
+      <c r="C5" t="n">
+        <v>26</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>37825</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>37826</v>
+      </c>
+      <c r="C6" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>37853</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>37854</v>
+      </c>
+      <c r="C7" t="n">
+        <v>22</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>37881</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>37882</v>
+      </c>
+      <c r="C8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>37916</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>37917</v>
+      </c>
+      <c r="C9" t="n">
+        <v>19</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>37944</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>37945</v>
+      </c>
+      <c r="C10" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>37972</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>37973</v>
+      </c>
+      <c r="C11" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>38091</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>38092</v>
+      </c>
+      <c r="C12" t="n">
+        <v>16</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>38245</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>38246</v>
+      </c>
+      <c r="C13" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>38280</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>38281</v>
+      </c>
+      <c r="C14" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>38308</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>38309</v>
+      </c>
+      <c r="C15" t="n">
+        <v>17.25</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>38336</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>38337</v>
+      </c>
+      <c r="C16" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>38371</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>38372</v>
+      </c>
+      <c r="C17" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>38399</v>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>38400</v>
+      </c>
+      <c r="C18" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>38427</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>38428</v>
+      </c>
+      <c r="C19" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>38462</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>38463</v>
+      </c>
+      <c r="C20" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>38490</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>38491</v>
+      </c>
+      <c r="C21" t="n">
+        <v>19.75</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>38609</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>38610</v>
+      </c>
+      <c r="C22" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>38644</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>38645</v>
+      </c>
+      <c r="C23" t="n">
+        <v>19</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>38679</v>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>38680</v>
+      </c>
+      <c r="C24" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>38700</v>
+      </c>
+      <c r="B25" s="1" t="n">
+        <v>38701</v>
+      </c>
+      <c r="C25" t="n">
+        <v>18</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>38735</v>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>38736</v>
+      </c>
+      <c r="C26" t="n">
+        <v>17.25</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.75</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>38784</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>38785</v>
+      </c>
+      <c r="C27" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.75</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>38826</v>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>38827</v>
+      </c>
+      <c r="C28" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.75</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>38868</v>
+      </c>
+      <c r="B29" s="1" t="n">
+        <v>38869</v>
+      </c>
+      <c r="C29" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>38917</v>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>38918</v>
+      </c>
+      <c r="C30" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="D30" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>38959</v>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>38960</v>
+      </c>
+      <c r="C31" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>39008</v>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>39009</v>
+      </c>
+      <c r="C32" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>39050</v>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>39051</v>
+      </c>
+      <c r="C33" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>39106</v>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>39107</v>
+      </c>
+      <c r="C34" t="n">
+        <v>13</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>39148</v>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>39149</v>
+      </c>
+      <c r="C35" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>39190</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>39191</v>
+      </c>
+      <c r="C36" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>39239</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>39240</v>
+      </c>
+      <c r="C37" t="n">
+        <v>12</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>39281</v>
+      </c>
+      <c r="B38" s="1" t="n">
+        <v>39282</v>
+      </c>
+      <c r="C38" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D38" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>39330</v>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>39331</v>
+      </c>
+      <c r="C39" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>39554</v>
+      </c>
+      <c r="B40" s="1" t="n">
+        <v>39555</v>
+      </c>
+      <c r="C40" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>39603</v>
+      </c>
+      <c r="B41" s="1" t="n">
+        <v>39604</v>
+      </c>
+      <c r="C41" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>39652</v>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>39653</v>
+      </c>
+      <c r="C42" t="n">
+        <v>13</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>39701</v>
+      </c>
+      <c r="B43" s="1" t="n">
+        <v>39702</v>
+      </c>
+      <c r="C43" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>39834</v>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>39835</v>
+      </c>
+      <c r="C44" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>39883</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>39884</v>
+      </c>
+      <c r="C45" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>39932</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>39933</v>
+      </c>
+      <c r="C46" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>39974</v>
+      </c>
+      <c r="B47" s="1" t="n">
+        <v>39975</v>
+      </c>
+      <c r="C47" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>40016</v>
+      </c>
+      <c r="B48" s="1" t="n">
+        <v>40017</v>
+      </c>
+      <c r="C48" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>40296</v>
+      </c>
+      <c r="B49" s="1" t="n">
+        <v>40297</v>
+      </c>
+      <c r="C49" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>40338</v>
+      </c>
+      <c r="B50" s="1" t="n">
+        <v>40339</v>
+      </c>
+      <c r="C50" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>40380</v>
+      </c>
+      <c r="B51" s="1" t="n">
+        <v>40381</v>
+      </c>
+      <c r="C51" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>40562</v>
+      </c>
+      <c r="B52" s="1" t="n">
+        <v>40563</v>
+      </c>
+      <c r="C52" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>40604</v>
+      </c>
+      <c r="B53" s="1" t="n">
+        <v>40605</v>
+      </c>
+      <c r="C53" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>selic_ini</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>selic_fim</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>selic_media</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>selic_max</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>selic_min</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>delta_pp</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sentido</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C2" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.51</v>
+      </c>
+      <c r="E2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>queda</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="D3" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="F3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="C4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D4" t="n">
+        <v>19.14</v>
+      </c>
+      <c r="E4" t="n">
+        <v>19.75</v>
+      </c>
+      <c r="F4" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15.32</v>
+      </c>
+      <c r="E5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-4.75</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>queda</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="C6" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="E6" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>queda</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="E7" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="F7" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="E8" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>queda</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="D9" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>selic_ini</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>selic_fim</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>selic_media</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>selic_max</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>selic_min</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>delta_selic_pp</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sentido_selic</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>tesouro_nacional</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>titulos_publicos</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>setor_externo</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>demais_operacoes</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>var_base</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ciclo_selic</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>instrumento_dominante</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>leitura</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C2" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>23.51</v>
+      </c>
+      <c r="E2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>queda</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>-1064</v>
+      </c>
+      <c r="J2" t="n">
+        <v>11181</v>
+      </c>
+      <c r="K2" t="n">
+        <v>643</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-10843</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-83</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Queda após pico (26,50% em fev.)</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Preço (Selic) + demais</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Copom herda 25% e sobe até 26,50% em fevereiro para ancorar a inflação de 2003; depois corta 10 pp, a 16,50% em dezembro. A base quase não se move (−83 milhões). Tesouro ainda é quase neutro; títulos injetam 11,2 bi e demais contraem 10,8 bi. O setor externo ainda não é o choque — o ajuste é de preço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="D3" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="F3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>-42140</v>
+      </c>
+      <c r="J3" t="n">
+        <v>52111</v>
+      </c>
+      <c r="K3" t="n">
+        <v>12599</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-8468</v>
+      </c>
+      <c r="M3" t="n">
+        <v>14102</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Alta do ciclo 2004–05 (16,00 → 17,75%)</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Títulos + Tesouro</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Selic pausa em 16% em abril e retoma a alta no segundo semestre. O Tesouro vira dreno estrutural (−42,1 bi). O setor externo começa a expandir (+12,6 bi). Títulos injetam 52,1 bi — mais do que compensam Tesouro e demais. A quantidade já cresce (+14,1 bi) enquanto o preço volta a apertar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="C4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D4" t="n">
+        <v>19.14</v>
+      </c>
+      <c r="E4" t="n">
+        <v>19.75</v>
+      </c>
+      <c r="F4" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>-43008</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2808</v>
+      </c>
+      <c r="K4" t="n">
+        <v>52395</v>
+      </c>
+      <c r="L4" t="n">
+        <v>319</v>
+      </c>
+      <c r="M4" t="n">
+        <v>12514</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Aperto máximo (pico 19,75%), depois corte</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Preço (Selic) + Tesouro; externo lidera a quantidade</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Média anual mais alta do período (19,14%). O aperto é quase só via juros: títulos quase somem (+2,8 bi). Quem expande a base é o setor externo (+52,4 bi); o Tesouro drena 43,0 bi. A quantidade cresce apesar da Selic no teto do ciclo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15.32</v>
+      </c>
+      <c r="E5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-4.75</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>queda</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>-59511</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-687</v>
+      </c>
+      <c r="K5" t="n">
+        <v>74369</v>
+      </c>
+      <c r="L5" t="n">
+        <v>5683</v>
+      </c>
+      <c r="M5" t="n">
+        <v>19854</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Corte contínuo (18,00 → 13,25%) — janela do gráfico TCU</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Externo expansionista; títulos neutros</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Começa a janela do gráfico da p. 33. Copom corta 4,75 pp. Títulos deixam de injetar (−0,7 bi). Externo acelera (+74,4 bi) e o Tesouro drena 59,5 bi. Política de juros em afrouxamento com absorção cambial sem repos líquidos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="C6" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="E6" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>queda</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>-55600</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-73974</v>
+      </c>
+      <c r="K6" t="n">
+        <v>155390</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-300</v>
+      </c>
+      <c r="M6" t="n">
+        <v>25516</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Queda ao piso pré-crise (11,25%)</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Esterilização clássica via títulos</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Caso-escola do cotejamento. Selic ainda cai (13,25 → 11,25%) enquanto o setor externo injeta o recorde da série (+155,4 bi). Títulos contraem 74,0 bi para que a overnight efetiva possa sentar na meta. Sem essa esterilização a base teria crescido cerca de 100 bi; cresceu 25,5 bi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="E7" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="F7" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>-74312</v>
+      </c>
+      <c r="J7" t="n">
+        <v>34059</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-12124</v>
+      </c>
+      <c r="L7" t="n">
+        <v>53311</v>
+      </c>
+      <c r="M7" t="n">
+        <v>933</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Alta a 13,75%; depois crise com Selic ainda alta</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Demais (compulsório) — instrumento secundário da p. 33</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>No primeiro semestre a Selic sobe 2,50 pp e o Tesouro faz a maior drenagem da série (−74,3 bi). No segundo, o externo inverte (−12,1 bi, único ano) e o Bacen injeta via demais (+53,3 bi, corte de compulsório) e títulos (+34,1 bi). A base quase não cresce (+0,9 bi). Assincronia: o preço permanece alto (13,75% até janeiro de 2009) enquanto a quantidade já é de socorro — exatamente o uso secundário que o TCU descreve nas pp. 32–33.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="E8" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>queda</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>-52312</v>
+      </c>
+      <c r="J8" t="n">
+        <v>11281</v>
+      </c>
+      <c r="K8" t="n">
+        <v>62937</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-3383</v>
+      </c>
+      <c r="M8" t="n">
+        <v>18523</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Corte agressivo ao piso de 8,75%</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Preço (Selic) + volta do externo</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Maior corte do período (−5,00 pp). O TCU lê o gráfico da p. 33 como o estímulo da crise. Externo volta (+62,9 bi). Títulos expandem pouco (+11,3 bi) com o estoque de compromissadas em 427,9 bi em dezembro. Demais deixa de injetar. Preço muito baixo e quantidade de novo liderada pelo câmbio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="D9" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="F9" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>-51204</v>
+      </c>
+      <c r="J9" t="n">
+        <v>249513</v>
+      </c>
+      <c r="K9" t="n">
+        <v>75553</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-233082</v>
+      </c>
+      <c r="M9" t="n">
+        <v>40780</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Alta tardia (8,75 → 10,75%); troca de instrumento</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Compulsório à frente da Selic; títulos como contrapartida</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Tese do TCU na p. 33: retirada intempestiva do estímulo. A Selic só sobe em 29/4 (9,50%), 10/6 (10,25%) e 22/7 (10,75%) e para aí, com IPCA em 5,91%. O compulsório aperta antes e mais forte (depósitos IF −236,9 bi; demais −233,1 bi). Títulos +249,5 bi não são afrouxamento: o TCU (p. 34) diz que a alta do compulsório 'abriu espaço' para resgatar repos (427,9 → 259,2 bi). A base ainda cresce 24,6% porque o externo (+75,6 bi) supera o Tesouro (−51,2 bi).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>evento</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>leitura_tcu_p33</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>oficial_copom</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Piso de 8,75% a.a.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>vigente até a reunião de 22/7/2009</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>corte para 8,75% na reunião de 22/7/2009, vigente em 23/7/2009; piso até 28/4/2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Selic em 10,25% a.a.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>aumentou para 10,25% apenas em 1º/9/2010</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10,25% vigente desde 10/6/2010 (reunião de 9/6); em 1º/9/2010 a meta já era 10,75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Alta de 0,50 pp para 11,25%</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>reunião de 19/1/2011</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>reunião de 19/1/2011, vigente em 20/1/2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Janela do gráfico da p. 33</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>janeiro de 2006 a março de 2011</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>o quadro da p. 35 começa em 2003; o cotejamento usa a série oficial 2003–2010 e marca a janela do gráfico</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Cruza reservas (TCU p. 43) com M1–M4, Selic e compromissadas
O salto do setor externo (R$ 0,6 bi em 2003 → R$ 155,4 bi em 2007) é
o fluxo em reais da compra de reservas, ativo do Bacen. A série oficial
M1–M4 mostra que essa emissão foi esterilizada na overnight e reciclou
para a liquidez ampla (M3), não para um M1 descontrolado.

Co-authored-by: cafla19791 <cafla19791@gmail.com>
</commit_message>
<xml_diff>
--- a/output/TCU_CG_2010.xlsx
+++ b/output/TCU_CG_2010.xlsx
@@ -31,7 +31,10 @@
     <sheet name="Selic_Anual" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="Cotejamento_Selic_Base" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="Selic_TCU_vs_oficial" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Base_Monetaria_IPCA" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Reservas_Internacionais" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Agregados_M1_M4" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Reservas_vs_M1M4" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Base_Monetaria_IPCA" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6499,6 +6502,1630 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>reservas_usd_mi</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ptax_fim</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>reservas_r_mi</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>delta_usd_mi</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>delta_r_mi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B2" t="n">
+        <v>37823</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.5333</v>
+      </c>
+      <c r="D2" t="n">
+        <v>133640.0059</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B3" t="n">
+        <v>49296</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.8892</v>
+      </c>
+      <c r="D3" t="n">
+        <v>142426.0032</v>
+      </c>
+      <c r="E3" t="n">
+        <v>11473</v>
+      </c>
+      <c r="F3" t="n">
+        <v>8785.997299999988</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B4" t="n">
+        <v>52935</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.6544</v>
+      </c>
+      <c r="D4" t="n">
+        <v>140510.664</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3639</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-1915.339200000017</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B5" t="n">
+        <v>53799</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.3407</v>
+      </c>
+      <c r="D5" t="n">
+        <v>125927.3193</v>
+      </c>
+      <c r="E5" t="n">
+        <v>864</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-14583.34469999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B6" t="n">
+        <v>85839</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.138</v>
+      </c>
+      <c r="D6" t="n">
+        <v>183523.782</v>
+      </c>
+      <c r="E6" t="n">
+        <v>32040</v>
+      </c>
+      <c r="F6" t="n">
+        <v>57596.46269999997</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B7" t="n">
+        <v>180334</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.7713</v>
+      </c>
+      <c r="D7" t="n">
+        <v>319425.6142</v>
+      </c>
+      <c r="E7" t="n">
+        <v>94495</v>
+      </c>
+      <c r="F7" t="n">
+        <v>135901.8322</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B8" t="n">
+        <v>193783</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.337</v>
+      </c>
+      <c r="D8" t="n">
+        <v>452870.871</v>
+      </c>
+      <c r="E8" t="n">
+        <v>13449</v>
+      </c>
+      <c r="F8" t="n">
+        <v>133445.2568</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B9" t="n">
+        <v>238520</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.7412</v>
+      </c>
+      <c r="D9" t="n">
+        <v>415311.024</v>
+      </c>
+      <c r="E9" t="n">
+        <v>44737</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-37559.84700000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B10" t="n">
+        <v>288575</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.6662</v>
+      </c>
+      <c r="D10" t="n">
+        <v>480823.665</v>
+      </c>
+      <c r="E10" t="n">
+        <v>50055</v>
+      </c>
+      <c r="F10" t="n">
+        <v>65512.64099999995</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>m1_restrito</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>m1</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>m4</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>var_base</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>var_base_pct</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>var_m1_restrito</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>var_m1_restrito_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>var_m1</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>var_m1_pct</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>var_m2</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>var_m2_pct</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>var_m3</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>var_m3_pct</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>var_m4</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>var_m4_pct</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>m3_menos_m2</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>m2_menos_m1</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>mult_m1</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>mult_m3</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>mult_m4</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B2" t="n">
+        <v>73302</v>
+      </c>
+      <c r="C2" t="n">
+        <v>69901</v>
+      </c>
+      <c r="D2" t="n">
+        <v>110334</v>
+      </c>
+      <c r="E2" t="n">
+        <v>400342</v>
+      </c>
+      <c r="F2" t="n">
+        <v>691108</v>
+      </c>
+      <c r="G2" t="n">
+        <v>800036</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>290766</v>
+      </c>
+      <c r="U2" t="n">
+        <v>290008</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1.505197675370386</v>
+      </c>
+      <c r="W2" t="n">
+        <v>9.428228424872446</v>
+      </c>
+      <c r="X2" t="n">
+        <v>10.91424517748493</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B3" t="n">
+        <v>73219</v>
+      </c>
+      <c r="C3" t="n">
+        <v>70802</v>
+      </c>
+      <c r="D3" t="n">
+        <v>112766</v>
+      </c>
+      <c r="E3" t="n">
+        <v>416248</v>
+      </c>
+      <c r="F3" t="n">
+        <v>841738</v>
+      </c>
+      <c r="G3" t="n">
+        <v>953805</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-83</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.1132301983574835</v>
+      </c>
+      <c r="J3" t="n">
+        <v>901</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1.288965823092658</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2432</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2.204216288723337</v>
+      </c>
+      <c r="N3" t="n">
+        <v>15906</v>
+      </c>
+      <c r="O3" t="n">
+        <v>3.973102996937627</v>
+      </c>
+      <c r="P3" t="n">
+        <v>150630</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>21.79543573508047</v>
+      </c>
+      <c r="R3" t="n">
+        <v>153769</v>
+      </c>
+      <c r="S3" t="n">
+        <v>19.22026008829603</v>
+      </c>
+      <c r="T3" t="n">
+        <v>425490</v>
+      </c>
+      <c r="U3" t="n">
+        <v>303482</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1.540119367923626</v>
+      </c>
+      <c r="W3" t="n">
+        <v>11.49616902716508</v>
+      </c>
+      <c r="X3" t="n">
+        <v>13.02674169273003</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B4" t="n">
+        <v>88733</v>
+      </c>
+      <c r="C4" t="n">
+        <v>87344</v>
+      </c>
+      <c r="D4" t="n">
+        <v>129660</v>
+      </c>
+      <c r="E4" t="n">
+        <v>495043</v>
+      </c>
+      <c r="F4" t="n">
+        <v>990548</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1104058</v>
+      </c>
+      <c r="H4" t="n">
+        <v>15514</v>
+      </c>
+      <c r="I4" t="n">
+        <v>21.18848932654092</v>
+      </c>
+      <c r="J4" t="n">
+        <v>16542</v>
+      </c>
+      <c r="K4" t="n">
+        <v>23.36374678681392</v>
+      </c>
+      <c r="L4" t="n">
+        <v>16894</v>
+      </c>
+      <c r="M4" t="n">
+        <v>14.98146604472979</v>
+      </c>
+      <c r="N4" t="n">
+        <v>78795</v>
+      </c>
+      <c r="O4" t="n">
+        <v>18.9298206838231</v>
+      </c>
+      <c r="P4" t="n">
+        <v>148810</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>17.67889770926345</v>
+      </c>
+      <c r="R4" t="n">
+        <v>150253</v>
+      </c>
+      <c r="S4" t="n">
+        <v>15.75301031133198</v>
+      </c>
+      <c r="T4" t="n">
+        <v>495505</v>
+      </c>
+      <c r="U4" t="n">
+        <v>365383</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1.461237645520832</v>
+      </c>
+      <c r="W4" t="n">
+        <v>11.16324253659856</v>
+      </c>
+      <c r="X4" t="n">
+        <v>12.44247348787937</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B5" t="n">
+        <v>101247</v>
+      </c>
+      <c r="C5" t="n">
+        <v>98306</v>
+      </c>
+      <c r="D5" t="n">
+        <v>146745</v>
+      </c>
+      <c r="E5" t="n">
+        <v>580696</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1166453</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1298801</v>
+      </c>
+      <c r="H5" t="n">
+        <v>12514</v>
+      </c>
+      <c r="I5" t="n">
+        <v>14.10298310662323</v>
+      </c>
+      <c r="J5" t="n">
+        <v>10962</v>
+      </c>
+      <c r="K5" t="n">
+        <v>12.55037552665323</v>
+      </c>
+      <c r="L5" t="n">
+        <v>17085</v>
+      </c>
+      <c r="M5" t="n">
+        <v>13.17677001388247</v>
+      </c>
+      <c r="N5" t="n">
+        <v>85653</v>
+      </c>
+      <c r="O5" t="n">
+        <v>17.30213335003221</v>
+      </c>
+      <c r="P5" t="n">
+        <v>175905</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>17.75835194256108</v>
+      </c>
+      <c r="R5" t="n">
+        <v>194743</v>
+      </c>
+      <c r="S5" t="n">
+        <v>17.63883781468003</v>
+      </c>
+      <c r="T5" t="n">
+        <v>585757</v>
+      </c>
+      <c r="U5" t="n">
+        <v>433951</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1.449376277815639</v>
+      </c>
+      <c r="W5" t="n">
+        <v>11.52086481574763</v>
+      </c>
+      <c r="X5" t="n">
+        <v>12.82804428773198</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B6" t="n">
+        <v>121102</v>
+      </c>
+      <c r="C6" t="n">
+        <v>118304</v>
+      </c>
+      <c r="D6" t="n">
+        <v>176890</v>
+      </c>
+      <c r="E6" t="n">
+        <v>657427</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1365958</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1506072</v>
+      </c>
+      <c r="H6" t="n">
+        <v>19855</v>
+      </c>
+      <c r="I6" t="n">
+        <v>19.61045759380524</v>
+      </c>
+      <c r="J6" t="n">
+        <v>19998</v>
+      </c>
+      <c r="K6" t="n">
+        <v>20.34260370679308</v>
+      </c>
+      <c r="L6" t="n">
+        <v>30145</v>
+      </c>
+      <c r="M6" t="n">
+        <v>20.5424375617568</v>
+      </c>
+      <c r="N6" t="n">
+        <v>76731</v>
+      </c>
+      <c r="O6" t="n">
+        <v>13.21362640693238</v>
+      </c>
+      <c r="P6" t="n">
+        <v>199505</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>17.10356096645129</v>
+      </c>
+      <c r="R6" t="n">
+        <v>207271</v>
+      </c>
+      <c r="S6" t="n">
+        <v>15.95864185506479</v>
+      </c>
+      <c r="T6" t="n">
+        <v>708531</v>
+      </c>
+      <c r="U6" t="n">
+        <v>480537</v>
+      </c>
+      <c r="V6" t="n">
+        <v>1.460669518257337</v>
+      </c>
+      <c r="W6" t="n">
+        <v>11.2794008356592</v>
+      </c>
+      <c r="X6" t="n">
+        <v>12.43639246255223</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B7" t="n">
+        <v>146617</v>
+      </c>
+      <c r="C7" t="n">
+        <v>143642</v>
+      </c>
+      <c r="D7" t="n">
+        <v>235075</v>
+      </c>
+      <c r="E7" t="n">
+        <v>779566</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1600006</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1827748</v>
+      </c>
+      <c r="H7" t="n">
+        <v>25515</v>
+      </c>
+      <c r="I7" t="n">
+        <v>21.06901620121882</v>
+      </c>
+      <c r="J7" t="n">
+        <v>25338</v>
+      </c>
+      <c r="K7" t="n">
+        <v>21.41770354341357</v>
+      </c>
+      <c r="L7" t="n">
+        <v>58185</v>
+      </c>
+      <c r="M7" t="n">
+        <v>32.89332353439991</v>
+      </c>
+      <c r="N7" t="n">
+        <v>122139</v>
+      </c>
+      <c r="O7" t="n">
+        <v>18.5783364540854</v>
+      </c>
+      <c r="P7" t="n">
+        <v>234048</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>17.13434820104278</v>
+      </c>
+      <c r="R7" t="n">
+        <v>321676</v>
+      </c>
+      <c r="S7" t="n">
+        <v>21.35860702542773</v>
+      </c>
+      <c r="T7" t="n">
+        <v>820440</v>
+      </c>
+      <c r="U7" t="n">
+        <v>544491</v>
+      </c>
+      <c r="V7" t="n">
+        <v>1.603327035746196</v>
+      </c>
+      <c r="W7" t="n">
+        <v>10.91282729833512</v>
+      </c>
+      <c r="X7" t="n">
+        <v>12.46613967002462</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B8" t="n">
+        <v>147550</v>
+      </c>
+      <c r="C8" t="n">
+        <v>145742</v>
+      </c>
+      <c r="D8" t="n">
+        <v>227167</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1086785</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1894809</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2165027</v>
+      </c>
+      <c r="H8" t="n">
+        <v>933</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.6363518555147163</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2100</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.461967948093168</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-7908</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-3.364032755503565</v>
+      </c>
+      <c r="N8" t="n">
+        <v>307219</v>
+      </c>
+      <c r="O8" t="n">
+        <v>39.40897884207366</v>
+      </c>
+      <c r="P8" t="n">
+        <v>294803</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>18.42511840580599</v>
+      </c>
+      <c r="R8" t="n">
+        <v>337279</v>
+      </c>
+      <c r="S8" t="n">
+        <v>18.45325504391195</v>
+      </c>
+      <c r="T8" t="n">
+        <v>808024</v>
+      </c>
+      <c r="U8" t="n">
+        <v>859618</v>
+      </c>
+      <c r="V8" t="n">
+        <v>1.539593358183666</v>
+      </c>
+      <c r="W8" t="n">
+        <v>12.84180955608268</v>
+      </c>
+      <c r="X8" t="n">
+        <v>14.6731751948492</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B9" t="n">
+        <v>166073</v>
+      </c>
+      <c r="C9" t="n">
+        <v>167400</v>
+      </c>
+      <c r="D9" t="n">
+        <v>254714</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1185866</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2196530</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2497479</v>
+      </c>
+      <c r="H9" t="n">
+        <v>18523</v>
+      </c>
+      <c r="I9" t="n">
+        <v>12.55371060657404</v>
+      </c>
+      <c r="J9" t="n">
+        <v>21658</v>
+      </c>
+      <c r="K9" t="n">
+        <v>14.86050692319303</v>
+      </c>
+      <c r="L9" t="n">
+        <v>27547</v>
+      </c>
+      <c r="M9" t="n">
+        <v>12.12632116460577</v>
+      </c>
+      <c r="N9" t="n">
+        <v>99081</v>
+      </c>
+      <c r="O9" t="n">
+        <v>9.116890645343844</v>
+      </c>
+      <c r="P9" t="n">
+        <v>301721</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>15.92355746674203</v>
+      </c>
+      <c r="R9" t="n">
+        <v>332452</v>
+      </c>
+      <c r="S9" t="n">
+        <v>15.35555907616857</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1010664</v>
+      </c>
+      <c r="U9" t="n">
+        <v>931152</v>
+      </c>
+      <c r="V9" t="n">
+        <v>1.533747207553305</v>
+      </c>
+      <c r="W9" t="n">
+        <v>13.22629205229026</v>
+      </c>
+      <c r="X9" t="n">
+        <v>15.03844092658048</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B10" t="n">
+        <v>206853</v>
+      </c>
+      <c r="C10" t="n">
+        <v>197388</v>
+      </c>
+      <c r="D10" t="n">
+        <v>287739</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1387912</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2681421</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2976783</v>
+      </c>
+      <c r="H10" t="n">
+        <v>40780</v>
+      </c>
+      <c r="I10" t="n">
+        <v>24.55546657192922</v>
+      </c>
+      <c r="J10" t="n">
+        <v>29988</v>
+      </c>
+      <c r="K10" t="n">
+        <v>17.91397849462366</v>
+      </c>
+      <c r="L10" t="n">
+        <v>33025</v>
+      </c>
+      <c r="M10" t="n">
+        <v>12.96552211499957</v>
+      </c>
+      <c r="N10" t="n">
+        <v>202046</v>
+      </c>
+      <c r="O10" t="n">
+        <v>17.03784407344506</v>
+      </c>
+      <c r="P10" t="n">
+        <v>484891</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>22.07531879828639</v>
+      </c>
+      <c r="R10" t="n">
+        <v>479304</v>
+      </c>
+      <c r="S10" t="n">
+        <v>19.1915127214283</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1293509</v>
+      </c>
+      <c r="U10" t="n">
+        <v>1100173</v>
+      </c>
+      <c r="V10" t="n">
+        <v>1.391031312091195</v>
+      </c>
+      <c r="W10" t="n">
+        <v>12.96293019680643</v>
+      </c>
+      <c r="X10" t="n">
+        <v>14.39081376629781</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>reservas_usd_mi</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ptax_fim</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>reservas_r_mi</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>setor_externo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>titulos_publicos</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>var_base</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>m1_restrito</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>m1</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>m4</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>m3_menos_m2</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>mult_m1</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>mult_m3</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>compromissadas</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>selic_fim</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>selic_media</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B2" t="n">
+        <v>37823</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.5333</v>
+      </c>
+      <c r="D2" t="n">
+        <v>133640.0059</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>73302</v>
+      </c>
+      <c r="I2" t="n">
+        <v>69901</v>
+      </c>
+      <c r="J2" t="n">
+        <v>110334</v>
+      </c>
+      <c r="K2" t="n">
+        <v>400342</v>
+      </c>
+      <c r="L2" t="n">
+        <v>691108</v>
+      </c>
+      <c r="M2" t="n">
+        <v>800036</v>
+      </c>
+      <c r="N2" t="n">
+        <v>290766</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1.505197675370386</v>
+      </c>
+      <c r="P2" t="n">
+        <v>9.428228424872446</v>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B3" t="n">
+        <v>49296</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.8892</v>
+      </c>
+      <c r="D3" t="n">
+        <v>142426.0032</v>
+      </c>
+      <c r="E3" t="n">
+        <v>643</v>
+      </c>
+      <c r="F3" t="n">
+        <v>11181</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-83</v>
+      </c>
+      <c r="H3" t="n">
+        <v>73219</v>
+      </c>
+      <c r="I3" t="n">
+        <v>70802</v>
+      </c>
+      <c r="J3" t="n">
+        <v>112766</v>
+      </c>
+      <c r="K3" t="n">
+        <v>416248</v>
+      </c>
+      <c r="L3" t="n">
+        <v>841738</v>
+      </c>
+      <c r="M3" t="n">
+        <v>953805</v>
+      </c>
+      <c r="N3" t="n">
+        <v>425490</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1.540119367923626</v>
+      </c>
+      <c r="P3" t="n">
+        <v>11.49616902716508</v>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="S3" t="n">
+        <v>23.51</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B4" t="n">
+        <v>52935</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.6544</v>
+      </c>
+      <c r="D4" t="n">
+        <v>140510.664</v>
+      </c>
+      <c r="E4" t="n">
+        <v>12599</v>
+      </c>
+      <c r="F4" t="n">
+        <v>52111</v>
+      </c>
+      <c r="G4" t="n">
+        <v>14102</v>
+      </c>
+      <c r="H4" t="n">
+        <v>88733</v>
+      </c>
+      <c r="I4" t="n">
+        <v>87344</v>
+      </c>
+      <c r="J4" t="n">
+        <v>129660</v>
+      </c>
+      <c r="K4" t="n">
+        <v>495043</v>
+      </c>
+      <c r="L4" t="n">
+        <v>990548</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1104058</v>
+      </c>
+      <c r="N4" t="n">
+        <v>495505</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1.461237645520832</v>
+      </c>
+      <c r="P4" t="n">
+        <v>11.16324253659856</v>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="S4" t="n">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B5" t="n">
+        <v>53799</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.3407</v>
+      </c>
+      <c r="D5" t="n">
+        <v>125927.3193</v>
+      </c>
+      <c r="E5" t="n">
+        <v>52395</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2808</v>
+      </c>
+      <c r="G5" t="n">
+        <v>12514</v>
+      </c>
+      <c r="H5" t="n">
+        <v>101247</v>
+      </c>
+      <c r="I5" t="n">
+        <v>98306</v>
+      </c>
+      <c r="J5" t="n">
+        <v>146745</v>
+      </c>
+      <c r="K5" t="n">
+        <v>580696</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1166453</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1298801</v>
+      </c>
+      <c r="N5" t="n">
+        <v>585757</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1.449376277815639</v>
+      </c>
+      <c r="P5" t="n">
+        <v>11.52086481574763</v>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="n">
+        <v>18</v>
+      </c>
+      <c r="S5" t="n">
+        <v>19.14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B6" t="n">
+        <v>85839</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.138</v>
+      </c>
+      <c r="D6" t="n">
+        <v>183523.782</v>
+      </c>
+      <c r="E6" t="n">
+        <v>74369</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-687</v>
+      </c>
+      <c r="G6" t="n">
+        <v>19854</v>
+      </c>
+      <c r="H6" t="n">
+        <v>121102</v>
+      </c>
+      <c r="I6" t="n">
+        <v>118304</v>
+      </c>
+      <c r="J6" t="n">
+        <v>176890</v>
+      </c>
+      <c r="K6" t="n">
+        <v>657427</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1365958</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1506072</v>
+      </c>
+      <c r="N6" t="n">
+        <v>708531</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1.460669518257337</v>
+      </c>
+      <c r="P6" t="n">
+        <v>11.2794008356592</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>60030</v>
+      </c>
+      <c r="R6" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="S6" t="n">
+        <v>15.32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B7" t="n">
+        <v>180334</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.7713</v>
+      </c>
+      <c r="D7" t="n">
+        <v>319425.6142</v>
+      </c>
+      <c r="E7" t="n">
+        <v>155390</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-73974</v>
+      </c>
+      <c r="G7" t="n">
+        <v>25516</v>
+      </c>
+      <c r="H7" t="n">
+        <v>146617</v>
+      </c>
+      <c r="I7" t="n">
+        <v>143642</v>
+      </c>
+      <c r="J7" t="n">
+        <v>235075</v>
+      </c>
+      <c r="K7" t="n">
+        <v>779566</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1600006</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1827748</v>
+      </c>
+      <c r="N7" t="n">
+        <v>820440</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1.603327035746196</v>
+      </c>
+      <c r="P7" t="n">
+        <v>10.91282729833512</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>165813</v>
+      </c>
+      <c r="R7" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="S7" t="n">
+        <v>12.04</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B8" t="n">
+        <v>193783</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.337</v>
+      </c>
+      <c r="D8" t="n">
+        <v>452870.871</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-12124</v>
+      </c>
+      <c r="F8" t="n">
+        <v>34059</v>
+      </c>
+      <c r="G8" t="n">
+        <v>933</v>
+      </c>
+      <c r="H8" t="n">
+        <v>147550</v>
+      </c>
+      <c r="I8" t="n">
+        <v>145742</v>
+      </c>
+      <c r="J8" t="n">
+        <v>227167</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1086785</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1894809</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2165027</v>
+      </c>
+      <c r="N8" t="n">
+        <v>808024</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1.539593358183666</v>
+      </c>
+      <c r="P8" t="n">
+        <v>12.84180955608268</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>300491</v>
+      </c>
+      <c r="R8" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="S8" t="n">
+        <v>12.45</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B9" t="n">
+        <v>238520</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.7412</v>
+      </c>
+      <c r="D9" t="n">
+        <v>415311.024</v>
+      </c>
+      <c r="E9" t="n">
+        <v>62937</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11281</v>
+      </c>
+      <c r="G9" t="n">
+        <v>18523</v>
+      </c>
+      <c r="H9" t="n">
+        <v>166073</v>
+      </c>
+      <c r="I9" t="n">
+        <v>167400</v>
+      </c>
+      <c r="J9" t="n">
+        <v>254714</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1185866</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2196530</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2497479</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1010664</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1.533747207553305</v>
+      </c>
+      <c r="P9" t="n">
+        <v>13.22629205229026</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>427874</v>
+      </c>
+      <c r="R9" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="S9" t="n">
+        <v>10.14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B10" t="n">
+        <v>288575</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.6662</v>
+      </c>
+      <c r="D10" t="n">
+        <v>480823.665</v>
+      </c>
+      <c r="E10" t="n">
+        <v>75553</v>
+      </c>
+      <c r="F10" t="n">
+        <v>249513</v>
+      </c>
+      <c r="G10" t="n">
+        <v>40780</v>
+      </c>
+      <c r="H10" t="n">
+        <v>206853</v>
+      </c>
+      <c r="I10" t="n">
+        <v>197388</v>
+      </c>
+      <c r="J10" t="n">
+        <v>287739</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1387912</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2681421</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2976783</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1293509</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1.391031312091195</v>
+      </c>
+      <c r="P10" t="n">
+        <v>12.96293019680643</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>259248</v>
+      </c>
+      <c r="R10" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="S10" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Explica por que a Selic não acelerou a queda após o superávit de 2003
A balança comercial e as reservas confirmam o fim da escassez de dólares.
A Selic, porém, já era o instrumento da meta de inflação, não o de fechar
o BP. O acumulado 2003–2016 (+459,7% na SGS 4390) é juro composto de um
nível ainda alto, com a conta corrente de volta ao déficit desde 2008.

Co-authored-by: cafla19791 <cafla19791@gmail.com>
</commit_message>
<xml_diff>
--- a/output/TCU_CG_2010.xlsx
+++ b/output/TCU_CG_2010.xlsx
@@ -34,7 +34,9 @@
     <sheet name="Reservas_Internacionais" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="Agregados_M1_M4" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="Reservas_vs_M1M4" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Base_Monetaria_IPCA" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Balanca_Comercial" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Selic_IPCA_2003_2016" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Base_Monetaria_IPCA" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8126,7 +8128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8137,67 +8139,350 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>tesouro_nacional</t>
+          <t>balanca</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>titulos_publicos</t>
+          <t>corrente</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>setor_externo</t>
+          <t>reservas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1995</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-4481</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1996</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-6601</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-7590</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-7596</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-2661</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-26784</v>
+      </c>
+      <c r="D6" t="n">
+        <v>36342</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-2169</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-26531</v>
+      </c>
+      <c r="D7" t="n">
+        <v>33011</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1224</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-24890</v>
+      </c>
+      <c r="D8" t="n">
+        <v>35866</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B9" t="n">
+        <v>11667</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-9407</v>
+      </c>
+      <c r="D9" t="n">
+        <v>37823</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B10" t="n">
+        <v>23341</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2193</v>
+      </c>
+      <c r="D10" t="n">
+        <v>49296</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B11" t="n">
+        <v>32106</v>
+      </c>
+      <c r="C11" t="n">
+        <v>8959</v>
+      </c>
+      <c r="D11" t="n">
+        <v>52935</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B12" t="n">
+        <v>43542</v>
+      </c>
+      <c r="C12" t="n">
+        <v>11679</v>
+      </c>
+      <c r="D12" t="n">
+        <v>53799</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B13" t="n">
+        <v>44519</v>
+      </c>
+      <c r="C13" t="n">
+        <v>10774</v>
+      </c>
+      <c r="D13" t="n">
+        <v>85839</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B14" t="n">
+        <v>37689</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-2754</v>
+      </c>
+      <c r="D14" t="n">
+        <v>180334</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B15" t="n">
+        <v>22040</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-35602</v>
+      </c>
+      <c r="D15" t="n">
+        <v>193783</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B16" t="n">
+        <v>22776</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-29328</v>
+      </c>
+      <c r="D16" t="n">
+        <v>238520</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B17" t="n">
+        <v>16462</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-86718</v>
+      </c>
+      <c r="D17" t="n">
+        <v>288575</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B18" t="n">
+        <v>25123</v>
+      </c>
+      <c r="C18" t="n">
+        <v>-83576</v>
+      </c>
+      <c r="D18" t="n">
+        <v>352012</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B19" t="n">
+        <v>14157</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-92678</v>
+      </c>
+      <c r="D19" t="n">
+        <v>373147</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-2390</v>
+      </c>
+      <c r="C20" t="n">
+        <v>-88384</v>
+      </c>
+      <c r="D20" t="n">
+        <v>358808</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-9148</v>
+      </c>
+      <c r="C21" t="n">
+        <v>-110494</v>
+      </c>
+      <c r="D21" t="n">
+        <v>363551</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B22" t="n">
+        <v>15022</v>
+      </c>
+      <c r="C22" t="n">
+        <v>-63409</v>
+      </c>
+      <c r="D22" t="n">
+        <v>356464</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B23" t="n">
+        <v>41544</v>
+      </c>
+      <c r="C23" t="n">
+        <v>-30529</v>
+      </c>
+      <c r="D23" t="n">
+        <v>365016</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>selic_pct</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ipca_pct</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>selic_acum_pct</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>demais_operacoes</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>var_base</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>identidade_ok</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>residuo</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>fator_ipca</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>tesouro_nacional_ipca</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>titulos_publicos_ipca</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>setor_externo_ipca</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>demais_operacoes_ipca</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>var_base_ipca</t>
+          <t>ipca_acum_pct</t>
         </is>
       </c>
     </row>
@@ -8206,43 +8491,16 @@
         <v>2003</v>
       </c>
       <c r="B2" t="n">
-        <v>-1064</v>
+        <v>23.33</v>
       </c>
       <c r="C2" t="n">
-        <v>11181</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>643</v>
+        <v>23.33</v>
       </c>
       <c r="E2" t="n">
-        <v>-10843</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-83</v>
-      </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>3.432404819188201</v>
-      </c>
-      <c r="J2" t="n">
-        <v>-3652.078727616245</v>
-      </c>
-      <c r="K2" t="n">
-        <v>38377.71828334327</v>
-      </c>
-      <c r="L2" t="n">
-        <v>2207.036298738013</v>
-      </c>
-      <c r="M2" t="n">
-        <v>-37217.56545445766</v>
-      </c>
-      <c r="N2" t="n">
-        <v>-284.8895999926207</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -8250,43 +8508,16 @@
         <v>2004</v>
       </c>
       <c r="B3" t="n">
-        <v>-42140</v>
+        <v>16.24</v>
       </c>
       <c r="C3" t="n">
-        <v>52111</v>
+        <v>7.6</v>
       </c>
       <c r="D3" t="n">
-        <v>12599</v>
+        <v>43.36</v>
       </c>
       <c r="E3" t="n">
-        <v>-8468</v>
-      </c>
-      <c r="F3" t="n">
-        <v>14102</v>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3.189948207730192</v>
-      </c>
-      <c r="J3" t="n">
-        <v>-134424.4174737503</v>
-      </c>
-      <c r="K3" t="n">
-        <v>166231.391053028</v>
-      </c>
-      <c r="L3" t="n">
-        <v>40190.15746919269</v>
-      </c>
-      <c r="M3" t="n">
-        <v>-27012.48142305926</v>
-      </c>
-      <c r="N3" t="n">
-        <v>44984.64962541117</v>
+        <v>17.61</v>
       </c>
     </row>
     <row r="4">
@@ -8294,43 +8525,16 @@
         <v>2005</v>
       </c>
       <c r="B4" t="n">
-        <v>-43008</v>
+        <v>19.04</v>
       </c>
       <c r="C4" t="n">
-        <v>2808</v>
+        <v>5.69</v>
       </c>
       <c r="D4" t="n">
-        <v>52395</v>
+        <v>70.66</v>
       </c>
       <c r="E4" t="n">
-        <v>319</v>
-      </c>
-      <c r="F4" t="n">
-        <v>12514</v>
-      </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>3.018219562813559</v>
-      </c>
-      <c r="J4" t="n">
-        <v>-129807.5869574855</v>
-      </c>
-      <c r="K4" t="n">
-        <v>8475.160532380472</v>
-      </c>
-      <c r="L4" t="n">
-        <v>158139.6139936164</v>
-      </c>
-      <c r="M4" t="n">
-        <v>962.8120405375251</v>
-      </c>
-      <c r="N4" t="n">
-        <v>37769.99960904887</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="5">
@@ -8338,43 +8542,16 @@
         <v>2006</v>
       </c>
       <c r="B5" t="n">
-        <v>-59511</v>
+        <v>15.08</v>
       </c>
       <c r="C5" t="n">
-        <v>-687</v>
+        <v>3.14</v>
       </c>
       <c r="D5" t="n">
-        <v>74369</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>5683</v>
-      </c>
-      <c r="F5" t="n">
-        <v>19854</v>
-      </c>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>2.9262823562432</v>
-      </c>
-      <c r="J5" t="n">
-        <v>-174145.9893023891</v>
-      </c>
-      <c r="K5" t="n">
-        <v>-2010.355978739078</v>
-      </c>
-      <c r="L5" t="n">
-        <v>217624.6925514505</v>
-      </c>
-      <c r="M5" t="n">
-        <v>16630.0626305301</v>
-      </c>
-      <c r="N5" t="n">
-        <v>58098.40990085249</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="6">
@@ -8382,43 +8559,16 @@
         <v>2007</v>
       </c>
       <c r="B6" t="n">
-        <v>-55600</v>
+        <v>11.84</v>
       </c>
       <c r="C6" t="n">
-        <v>-73974</v>
+        <v>4.46</v>
       </c>
       <c r="D6" t="n">
-        <v>155390</v>
+        <v>119.66</v>
       </c>
       <c r="E6" t="n">
-        <v>-300</v>
-      </c>
-      <c r="F6" t="n">
-        <v>25516</v>
-      </c>
-      <c r="G6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>2.801414074154887</v>
-      </c>
-      <c r="J6" t="n">
-        <v>-155758.6225230117</v>
-      </c>
-      <c r="K6" t="n">
-        <v>-207231.8047215336</v>
-      </c>
-      <c r="L6" t="n">
-        <v>435311.7329829279</v>
-      </c>
-      <c r="M6" t="n">
-        <v>-840.4242222464661</v>
-      </c>
-      <c r="N6" t="n">
-        <v>71480.8815161361</v>
+        <v>33.92</v>
       </c>
     </row>
     <row r="7">
@@ -8426,43 +8576,16 @@
         <v>2008</v>
       </c>
       <c r="B7" t="n">
-        <v>-74312</v>
+        <v>12.48</v>
       </c>
       <c r="C7" t="n">
-        <v>34059</v>
+        <v>5.9</v>
       </c>
       <c r="D7" t="n">
-        <v>-12124</v>
+        <v>147.08</v>
       </c>
       <c r="E7" t="n">
-        <v>53311</v>
-      </c>
-      <c r="F7" t="n">
-        <v>933</v>
-      </c>
-      <c r="G7" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>2.645281282109639</v>
-      </c>
-      <c r="J7" t="n">
-        <v>-196576.1426361315</v>
-      </c>
-      <c r="K7" t="n">
-        <v>90095.63518737219</v>
-      </c>
-      <c r="L7" t="n">
-        <v>-32071.39026429726</v>
-      </c>
-      <c r="M7" t="n">
-        <v>141022.590430547</v>
-      </c>
-      <c r="N7" t="n">
-        <v>2468.047436208293</v>
+        <v>41.82</v>
       </c>
     </row>
     <row r="8">
@@ -8470,43 +8593,16 @@
         <v>2009</v>
       </c>
       <c r="B8" t="n">
-        <v>-52312</v>
+        <v>9.92</v>
       </c>
       <c r="C8" t="n">
-        <v>11281</v>
+        <v>4.31</v>
       </c>
       <c r="D8" t="n">
-        <v>62937</v>
+        <v>171.6</v>
       </c>
       <c r="E8" t="n">
-        <v>-3383</v>
-      </c>
-      <c r="F8" t="n">
-        <v>18523</v>
-      </c>
-      <c r="G8" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>2.535931209916586</v>
-      </c>
-      <c r="J8" t="n">
-        <v>-132659.6334531564</v>
-      </c>
-      <c r="K8" t="n">
-        <v>28607.839979069</v>
-      </c>
-      <c r="L8" t="n">
-        <v>159603.9025585201</v>
-      </c>
-      <c r="M8" t="n">
-        <v>-8579.055283147809</v>
-      </c>
-      <c r="N8" t="n">
-        <v>46973.05380128491</v>
+        <v>47.94</v>
       </c>
     </row>
     <row r="9">
@@ -8514,43 +8610,118 @@
         <v>2010</v>
       </c>
       <c r="B9" t="n">
-        <v>-51204</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="C9" t="n">
-        <v>249513</v>
+        <v>5.91</v>
       </c>
       <c r="D9" t="n">
-        <v>75553</v>
+        <v>198.17</v>
       </c>
       <c r="E9" t="n">
-        <v>-233082</v>
-      </c>
-      <c r="F9" t="n">
-        <v>40780</v>
-      </c>
-      <c r="G9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>2.394441995846377</v>
-      </c>
-      <c r="J9" t="n">
-        <v>-122605.0079553179</v>
-      </c>
-      <c r="K9" t="n">
-        <v>597444.4057096171</v>
-      </c>
-      <c r="L9" t="n">
-        <v>180907.2761121813</v>
-      </c>
-      <c r="M9" t="n">
-        <v>-558101.3292758652</v>
-      </c>
-      <c r="N9" t="n">
-        <v>97645.34459061525</v>
+        <v>56.68</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B10" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="C10" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>232.81</v>
+      </c>
+      <c r="E10" t="n">
+        <v>66.87</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B11" t="n">
+        <v>8.48</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="D11" t="n">
+        <v>261.03</v>
+      </c>
+      <c r="E11" t="n">
+        <v>76.61</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B12" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="C12" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="D12" t="n">
+        <v>290.69</v>
+      </c>
+      <c r="E12" t="n">
+        <v>87.05</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B13" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="C13" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="D13" t="n">
+        <v>333.31</v>
+      </c>
+      <c r="E13" t="n">
+        <v>99.04000000000001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B14" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="C14" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="D14" t="n">
+        <v>390.88</v>
+      </c>
+      <c r="E14" t="n">
+        <v>120.28</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B15" t="n">
+        <v>14.03</v>
+      </c>
+      <c r="C15" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="D15" t="n">
+        <v>459.74</v>
+      </c>
+      <c r="E15" t="n">
+        <v>134.13</v>
       </c>
     </row>
   </sheetData>
@@ -9274,6 +9445,444 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tesouro_nacional</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>titulos_publicos</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>setor_externo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>demais_operacoes</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>var_base</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>identidade_ok</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>residuo</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>fator_ipca</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>tesouro_nacional_ipca</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>titulos_publicos_ipca</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>setor_externo_ipca</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>demais_operacoes_ipca</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>var_base_ipca</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-1064</v>
+      </c>
+      <c r="C2" t="n">
+        <v>11181</v>
+      </c>
+      <c r="D2" t="n">
+        <v>643</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-10843</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-83</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.432404819188201</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-3652.078727616245</v>
+      </c>
+      <c r="K2" t="n">
+        <v>38377.71828334327</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2207.036298738013</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-37217.56545445766</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-284.8895999926207</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-42140</v>
+      </c>
+      <c r="C3" t="n">
+        <v>52111</v>
+      </c>
+      <c r="D3" t="n">
+        <v>12599</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-8468</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14102</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3.189948207730192</v>
+      </c>
+      <c r="J3" t="n">
+        <v>-134424.4174737503</v>
+      </c>
+      <c r="K3" t="n">
+        <v>166231.391053028</v>
+      </c>
+      <c r="L3" t="n">
+        <v>40190.15746919269</v>
+      </c>
+      <c r="M3" t="n">
+        <v>-27012.48142305926</v>
+      </c>
+      <c r="N3" t="n">
+        <v>44984.64962541117</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-43008</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2808</v>
+      </c>
+      <c r="D4" t="n">
+        <v>52395</v>
+      </c>
+      <c r="E4" t="n">
+        <v>319</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12514</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.018219562813559</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-129807.5869574855</v>
+      </c>
+      <c r="K4" t="n">
+        <v>8475.160532380472</v>
+      </c>
+      <c r="L4" t="n">
+        <v>158139.6139936164</v>
+      </c>
+      <c r="M4" t="n">
+        <v>962.8120405375251</v>
+      </c>
+      <c r="N4" t="n">
+        <v>37769.99960904887</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-59511</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-687</v>
+      </c>
+      <c r="D5" t="n">
+        <v>74369</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5683</v>
+      </c>
+      <c r="F5" t="n">
+        <v>19854</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.9262823562432</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-174145.9893023891</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-2010.355978739078</v>
+      </c>
+      <c r="L5" t="n">
+        <v>217624.6925514505</v>
+      </c>
+      <c r="M5" t="n">
+        <v>16630.0626305301</v>
+      </c>
+      <c r="N5" t="n">
+        <v>58098.40990085249</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-55600</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-73974</v>
+      </c>
+      <c r="D6" t="n">
+        <v>155390</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-300</v>
+      </c>
+      <c r="F6" t="n">
+        <v>25516</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.801414074154887</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-155758.6225230117</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-207231.8047215336</v>
+      </c>
+      <c r="L6" t="n">
+        <v>435311.7329829279</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-840.4242222464661</v>
+      </c>
+      <c r="N6" t="n">
+        <v>71480.8815161361</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-74312</v>
+      </c>
+      <c r="C7" t="n">
+        <v>34059</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-12124</v>
+      </c>
+      <c r="E7" t="n">
+        <v>53311</v>
+      </c>
+      <c r="F7" t="n">
+        <v>933</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.645281282109639</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-196576.1426361315</v>
+      </c>
+      <c r="K7" t="n">
+        <v>90095.63518737219</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-32071.39026429726</v>
+      </c>
+      <c r="M7" t="n">
+        <v>141022.590430547</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2468.047436208293</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-52312</v>
+      </c>
+      <c r="C8" t="n">
+        <v>11281</v>
+      </c>
+      <c r="D8" t="n">
+        <v>62937</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-3383</v>
+      </c>
+      <c r="F8" t="n">
+        <v>18523</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.535931209916586</v>
+      </c>
+      <c r="J8" t="n">
+        <v>-132659.6334531564</v>
+      </c>
+      <c r="K8" t="n">
+        <v>28607.839979069</v>
+      </c>
+      <c r="L8" t="n">
+        <v>159603.9025585201</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-8579.055283147809</v>
+      </c>
+      <c r="N8" t="n">
+        <v>46973.05380128491</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-51204</v>
+      </c>
+      <c r="C9" t="n">
+        <v>249513</v>
+      </c>
+      <c r="D9" t="n">
+        <v>75553</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-233082</v>
+      </c>
+      <c r="F9" t="n">
+        <v>40780</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.394441995846377</v>
+      </c>
+      <c r="J9" t="n">
+        <v>-122605.0079553179</v>
+      </c>
+      <c r="K9" t="n">
+        <v>597444.4057096171</v>
+      </c>
+      <c r="L9" t="n">
+        <v>180907.2761121813</v>
+      </c>
+      <c r="M9" t="n">
+        <v>-558101.3292758652</v>
+      </c>
+      <c r="N9" t="n">
+        <v>97645.34459061525</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Simula a DBGG se indiretas, participações e três renúncias fossem à Conta Única
Monta o contrafactual 2003–2015 dos fatores da dívida bruta: desembolsos
indiretos do BNDES, participações acionárias da BNDESPAR e as famílias de
renúncia regional, inovação e imunes/isentas, como se tivessem ido à
Conta Única e evitado emissão de DPF.

Co-authored-by: cafla19791 <cafla19791@gmail.com>
</commit_message>
<xml_diff>
--- a/output/TCU_CG_2010.xlsx
+++ b/output/TCU_CG_2010.xlsx
@@ -36,7 +36,9 @@
     <sheet name="Reservas_vs_M1M4" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="Balanca_Comercial" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="Selic_IPCA_2003_2016" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Base_Monetaria_IPCA" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="DBGG_Fluxos_Conta_Unica" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="DBGG_Simulacao_Conta_Unica" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Base_Monetaria_IPCA" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9451,6 +9453,1346 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Q14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>indiretas</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>participacoes</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>participacoes_uso</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>regional_funcao</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>zfm_alc</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>regional_ampla</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>inovacao</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>imunes</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>renuncia</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fluxo_total</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>tesouro_captacao</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>tesouro_devolucao</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>pib</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>selic_pct</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>dbgg</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>dbgg_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>14546</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1690.247035900375</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6656.549323343208</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8346.796359243583</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>5588.723273031546</v>
+      </c>
+      <c r="J2" t="n">
+        <v>13935.51963227513</v>
+      </c>
+      <c r="K2" t="n">
+        <v>28481.51963227513</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1717950.4</v>
+      </c>
+      <c r="O2" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>19854</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1926.180850640625</v>
+      </c>
+      <c r="F3" t="n">
+        <v>7585.706447423833</v>
+      </c>
+      <c r="G3" t="n">
+        <v>9511.887298064457</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>6368.827466872989</v>
+      </c>
+      <c r="J3" t="n">
+        <v>15880.71476493745</v>
+      </c>
+      <c r="K3" t="n">
+        <v>35734.71476493745</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1957751.2</v>
+      </c>
+      <c r="O3" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>21009</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2135.582038513043</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8410.372490808964</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10545.95452932201</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>7061.202763031775</v>
+      </c>
+      <c r="J4" t="n">
+        <v>17607.15729235378</v>
+      </c>
+      <c r="K4" t="n">
+        <v>38616.15729235378</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2170584.5</v>
+      </c>
+      <c r="O4" t="n">
+        <v>19.04</v>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>25307</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2370.595537348141</v>
+      </c>
+      <c r="F5" t="n">
+        <v>9335.905216748028</v>
+      </c>
+      <c r="G5" t="n">
+        <v>11706.50075409617</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1363.099466475377</v>
+      </c>
+      <c r="I5" t="n">
+        <v>7838.263975102851</v>
+      </c>
+      <c r="J5" t="n">
+        <v>20907.8641956744</v>
+      </c>
+      <c r="K5" t="n">
+        <v>46214.8641956744</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>2409449.9</v>
+      </c>
+      <c r="O5" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1336644.9</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>55.48</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>32810</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1962.548</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1962.548</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2676.396421919258</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10540.21359773287</v>
+      </c>
+      <c r="G6" t="n">
+        <v>13216.61001965213</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1538.935882278673</v>
+      </c>
+      <c r="I6" t="n">
+        <v>8849.380388394384</v>
+      </c>
+      <c r="J6" t="n">
+        <v>23604.92629032519</v>
+      </c>
+      <c r="K6" t="n">
+        <v>58377.47429032519</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2720262.9</v>
+      </c>
+      <c r="O6" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1542851.83</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>56.72</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>42779</v>
+      </c>
+      <c r="C7" t="n">
+        <v>7901.455</v>
+      </c>
+      <c r="D7" t="n">
+        <v>7901.455</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3059.654965596676</v>
+      </c>
+      <c r="F7" t="n">
+        <v>12049.56657714659</v>
+      </c>
+      <c r="G7" t="n">
+        <v>15109.22154274326</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1759.310681850439</v>
+      </c>
+      <c r="I7" t="n">
+        <v>10116.60695181633</v>
+      </c>
+      <c r="J7" t="n">
+        <v>26985.13917641003</v>
+      </c>
+      <c r="K7" t="n">
+        <v>77665.59417641003</v>
+      </c>
+      <c r="L7" t="n">
+        <v>22500</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3109803.1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1740887.81</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>55.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>50409</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2746.931</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2746.931</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3279.291396532265</v>
+      </c>
+      <c r="F8" t="n">
+        <v>12914.54116646572</v>
+      </c>
+      <c r="G8" t="n">
+        <v>16193.83256299798</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1885.602281201784</v>
+      </c>
+      <c r="I8" t="n">
+        <v>10842.82460349909</v>
+      </c>
+      <c r="J8" t="n">
+        <v>28922.25944769886</v>
+      </c>
+      <c r="K8" t="n">
+        <v>82078.19044769886</v>
+      </c>
+      <c r="L8" t="n">
+        <v>105000</v>
+      </c>
+      <c r="M8" t="n">
+        <v>4080</v>
+      </c>
+      <c r="N8" t="n">
+        <v>3333039.4</v>
+      </c>
+      <c r="O8" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1973423.68</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>59.21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>81538</v>
+      </c>
+      <c r="C9" t="n">
+        <v>25429.091</v>
+      </c>
+      <c r="D9" t="n">
+        <v>25429.091</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3823.1845190131</v>
+      </c>
+      <c r="F9" t="n">
+        <v>15056.50699721321</v>
+      </c>
+      <c r="G9" t="n">
+        <v>18879.69151622631</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2198.342440116702</v>
+      </c>
+      <c r="I9" t="n">
+        <v>12641.1819365331</v>
+      </c>
+      <c r="J9" t="n">
+        <v>33719.21589287611</v>
+      </c>
+      <c r="K9" t="n">
+        <v>140686.3068928761</v>
+      </c>
+      <c r="L9" t="n">
+        <v>107100</v>
+      </c>
+      <c r="M9" t="n">
+        <v>10440</v>
+      </c>
+      <c r="N9" t="n">
+        <v>3885847</v>
+      </c>
+      <c r="O9" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2011521.66</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>51.77</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B10" t="n">
+        <v>69353</v>
+      </c>
+      <c r="C10" t="n">
+        <v>727.355</v>
+      </c>
+      <c r="D10" t="n">
+        <v>727.355</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4305.809238420245</v>
+      </c>
+      <c r="F10" t="n">
+        <v>16957.18493432138</v>
+      </c>
+      <c r="G10" t="n">
+        <v>21262.99417274163</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2475.853085508208</v>
+      </c>
+      <c r="I10" t="n">
+        <v>14236.95814214214</v>
+      </c>
+      <c r="J10" t="n">
+        <v>37975.80540039198</v>
+      </c>
+      <c r="K10" t="n">
+        <v>108056.160400392</v>
+      </c>
+      <c r="L10" t="n">
+        <v>50200</v>
+      </c>
+      <c r="M10" t="n">
+        <v>14560</v>
+      </c>
+      <c r="N10" t="n">
+        <v>4376382</v>
+      </c>
+      <c r="O10" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="P10" t="n">
+        <v>2243603.72</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>51.27</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B11" t="n">
+        <v>67109</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1603.942</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1603.942</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4737.118032378402</v>
+      </c>
+      <c r="F11" t="n">
+        <v>18655.76993378851</v>
+      </c>
+      <c r="G11" t="n">
+        <v>23392.88796616691</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2723.856921535071</v>
+      </c>
+      <c r="I11" t="n">
+        <v>15663.0606250689</v>
+      </c>
+      <c r="J11" t="n">
+        <v>41779.80551277089</v>
+      </c>
+      <c r="K11" t="n">
+        <v>110492.7475127709</v>
+      </c>
+      <c r="L11" t="n">
+        <v>55000</v>
+      </c>
+      <c r="M11" t="n">
+        <v>13310</v>
+      </c>
+      <c r="N11" t="n">
+        <v>4814760</v>
+      </c>
+      <c r="O11" t="n">
+        <v>8.48</v>
+      </c>
+      <c r="P11" t="n">
+        <v>2583946.35</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>53.67</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B12" t="n">
+        <v>97222</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2083.154</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2083.154</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5245.642255620488</v>
+      </c>
+      <c r="F12" t="n">
+        <v>20658.44557955445</v>
+      </c>
+      <c r="G12" t="n">
+        <v>25904.08783517493</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3016.259858463951</v>
+      </c>
+      <c r="I12" t="n">
+        <v>17344.4723364756</v>
+      </c>
+      <c r="J12" t="n">
+        <v>46264.82003011448</v>
+      </c>
+      <c r="K12" t="n">
+        <v>145569.9740301145</v>
+      </c>
+      <c r="L12" t="n">
+        <v>41000</v>
+      </c>
+      <c r="M12" t="n">
+        <v>14740</v>
+      </c>
+      <c r="N12" t="n">
+        <v>5331619</v>
+      </c>
+      <c r="O12" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="P12" t="n">
+        <v>2747996.71</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>51.54</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B13" t="n">
+        <v>85493</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1292.122</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1292.122</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5685.76262670772</v>
+      </c>
+      <c r="F13" t="n">
+        <v>22391.73242823669</v>
+      </c>
+      <c r="G13" t="n">
+        <v>28077.49505494441</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3269.330377480054</v>
+      </c>
+      <c r="I13" t="n">
+        <v>18799.70988967754</v>
+      </c>
+      <c r="J13" t="n">
+        <v>50146.53532210201</v>
+      </c>
+      <c r="K13" t="n">
+        <v>136931.657322102</v>
+      </c>
+      <c r="L13" t="n">
+        <v>60000</v>
+      </c>
+      <c r="M13" t="n">
+        <v>6200</v>
+      </c>
+      <c r="N13" t="n">
+        <v>5778953</v>
+      </c>
+      <c r="O13" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="P13" t="n">
+        <v>3252448.55</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>56.28</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B14" t="n">
+        <v>50946</v>
+      </c>
+      <c r="C14" t="n">
+        <v>666.136</v>
+      </c>
+      <c r="D14" t="n">
+        <v>666.136</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5899.1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>23231.9</v>
+      </c>
+      <c r="G14" t="n">
+        <v>29131</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3392</v>
+      </c>
+      <c r="I14" t="n">
+        <v>19505.1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>52028.1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>103640.236</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>24670</v>
+      </c>
+      <c r="N14" t="n">
+        <v>5995787</v>
+      </c>
+      <c r="O14" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="P14" t="n">
+        <v>3927523.06</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>65.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fluxo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>emissao_evitada</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>juros_evitados</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>acum_fluxo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>saldo_selic</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dbgg_oficial</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>dbgg_cf_estoque</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dbgg_cf_selic</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>dbgg_oficial_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dbgg_cf_estoque_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dbgg_cf_selic_pct</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>delta_oficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>28481.51963227513</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-28481.51963227513</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>28481.51963227513</v>
+      </c>
+      <c r="F2" t="n">
+        <v>28481.51963227513</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>35734.71476493745</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-35734.71476493745</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4625.398788281481</v>
+      </c>
+      <c r="E3" t="n">
+        <v>64216.23439721257</v>
+      </c>
+      <c r="F3" t="n">
+        <v>68841.63318549405</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>38616.15729235378</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-38616.15729235378</v>
+      </c>
+      <c r="D4" t="n">
+        <v>13107.44695851807</v>
+      </c>
+      <c r="E4" t="n">
+        <v>102832.3916895664</v>
+      </c>
+      <c r="F4" t="n">
+        <v>120565.2374363659</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>46214.8641956744</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-46214.8641956744</v>
+      </c>
+      <c r="D5" t="n">
+        <v>18181.23780540398</v>
+      </c>
+      <c r="E5" t="n">
+        <v>149047.2558852407</v>
+      </c>
+      <c r="F5" t="n">
+        <v>184961.3394374443</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1336644.9</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1187597.644114759</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1151683.560562556</v>
+      </c>
+      <c r="J5" t="n">
+        <v>55.48</v>
+      </c>
+      <c r="K5" t="n">
+        <v>49.28916115312293</v>
+      </c>
+      <c r="L5" t="n">
+        <v>47.79860998821995</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>58377.47429032519</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-58377.47429032519</v>
+      </c>
+      <c r="D6" t="n">
+        <v>21899.4225893934</v>
+      </c>
+      <c r="E6" t="n">
+        <v>207424.7301755659</v>
+      </c>
+      <c r="F6" t="n">
+        <v>265238.2363171629</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1542851.83</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1335427.099824434</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1277613.593682837</v>
+      </c>
+      <c r="J6" t="n">
+        <v>56.72</v>
+      </c>
+      <c r="K6" t="n">
+        <v>49.09183960948901</v>
+      </c>
+      <c r="L6" t="n">
+        <v>46.96654847892964</v>
+      </c>
+      <c r="M6" t="n">
+        <v>206206.9300000002</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>77665.59417641003</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-77665.59417641003</v>
+      </c>
+      <c r="D7" t="n">
+        <v>33101.73189238193</v>
+      </c>
+      <c r="E7" t="n">
+        <v>285090.3243519759</v>
+      </c>
+      <c r="F7" t="n">
+        <v>376005.5623859548</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1740887.81</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1455797.485648024</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1364882.247614045</v>
+      </c>
+      <c r="J7" t="n">
+        <v>55.98</v>
+      </c>
+      <c r="K7" t="n">
+        <v>46.81317237248957</v>
+      </c>
+      <c r="L7" t="n">
+        <v>43.88966772893259</v>
+      </c>
+      <c r="M7" t="n">
+        <v>198035.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>82078.19044769886</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-82078.19044769886</v>
+      </c>
+      <c r="D8" t="n">
+        <v>37299.75178868671</v>
+      </c>
+      <c r="E8" t="n">
+        <v>367168.5147996748</v>
+      </c>
+      <c r="F8" t="n">
+        <v>495383.5046223403</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1973423.68</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1606255.165200325</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1478040.175377659</v>
+      </c>
+      <c r="J8" t="n">
+        <v>59.21</v>
+      </c>
+      <c r="K8" t="n">
+        <v>48.19190451815017</v>
+      </c>
+      <c r="L8" t="n">
+        <v>44.34511561362459</v>
+      </c>
+      <c r="M8" t="n">
+        <v>232535.8699999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>140686.3068928761</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-140686.3068928761</v>
+      </c>
+      <c r="D9" t="n">
+        <v>48448.50675206488</v>
+      </c>
+      <c r="E9" t="n">
+        <v>507854.8216925509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>684518.3182672812</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2011521.66</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1503666.838307449</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1327003.341732719</v>
+      </c>
+      <c r="J9" t="n">
+        <v>51.77</v>
+      </c>
+      <c r="K9" t="n">
+        <v>38.69598670013125</v>
+      </c>
+      <c r="L9" t="n">
+        <v>34.14965493321581</v>
+      </c>
+      <c r="M9" t="n">
+        <v>38097.97999999998</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B10" t="n">
+        <v>108056.160400392</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-108056.160400392</v>
+      </c>
+      <c r="D10" t="n">
+        <v>79472.57675083134</v>
+      </c>
+      <c r="E10" t="n">
+        <v>615910.9820929428</v>
+      </c>
+      <c r="F10" t="n">
+        <v>872047.0554185046</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2243603.72</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1627692.737907057</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1371556.664581496</v>
+      </c>
+      <c r="J10" t="n">
+        <v>51.27</v>
+      </c>
+      <c r="K10" t="n">
+        <v>37.19265680891333</v>
+      </c>
+      <c r="L10" t="n">
+        <v>31.3399667712164</v>
+      </c>
+      <c r="M10" t="n">
+        <v>232082.0600000003</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B11" t="n">
+        <v>110492.7475127709</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-110492.7475127709</v>
+      </c>
+      <c r="D11" t="n">
+        <v>73949.59029948919</v>
+      </c>
+      <c r="E11" t="n">
+        <v>726403.7296057136</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1056489.393230765</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2583946.35</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1857542.620394286</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1527456.956769235</v>
+      </c>
+      <c r="J11" t="n">
+        <v>53.67</v>
+      </c>
+      <c r="K11" t="n">
+        <v>38.58017056705395</v>
+      </c>
+      <c r="L11" t="n">
+        <v>31.72446719606451</v>
+      </c>
+      <c r="M11" t="n">
+        <v>340342.6299999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B12" t="n">
+        <v>145569.9740301145</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-145569.9740301145</v>
+      </c>
+      <c r="D12" t="n">
+        <v>86737.77918424578</v>
+      </c>
+      <c r="E12" t="n">
+        <v>871973.7036358281</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1288797.146445125</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2747996.71</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1876023.006364172</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1459199.563554875</v>
+      </c>
+      <c r="J12" t="n">
+        <v>51.54</v>
+      </c>
+      <c r="K12" t="n">
+        <v>35.18674170761587</v>
+      </c>
+      <c r="L12" t="n">
+        <v>27.36878917182332</v>
+      </c>
+      <c r="M12" t="n">
+        <v>164050.3599999999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B13" t="n">
+        <v>136931.657322102</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-136931.657322102</v>
+      </c>
+      <c r="D13" t="n">
+        <v>140607.7686771631</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1008905.36095793</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1566336.57244439</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3252448.55</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2243543.18904207</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1686111.97755561</v>
+      </c>
+      <c r="J13" t="n">
+        <v>56.28</v>
+      </c>
+      <c r="K13" t="n">
+        <v>38.82265851689865</v>
+      </c>
+      <c r="L13" t="n">
+        <v>29.17677263607456</v>
+      </c>
+      <c r="M13" t="n">
+        <v>504451.8399999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B14" t="n">
+        <v>103640.236</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-103640.236</v>
+      </c>
+      <c r="D14" t="n">
+        <v>208166.1304778594</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1112545.59695793</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1878142.938922249</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3927523.06</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2814977.46304207</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2049380.121077751</v>
+      </c>
+      <c r="J14" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>46.94925725416981</v>
+      </c>
+      <c r="L14" t="n">
+        <v>34.18033564364028</v>
+      </c>
+      <c r="M14" t="n">
+        <v>675074.5100000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Aplica bloco macrométrico ao contrafactual da Conta Única
Solta o resto estático: o PIB reage ao corte de renúncia e de indiretas,
a receita residual vaza pela elasticidade IFI e a DBGG/PIB usa o
denominador já reduzido. A Macrométrica comercial não está acessível;
este é o sistema simultâneo da mesma classe.

Co-authored-by: cafla19791 <cafla19791@gmail.com>
</commit_message>
<xml_diff>
--- a/output/TCU_CG_2010.xlsx
+++ b/output/TCU_CG_2010.xlsx
@@ -38,7 +38,9 @@
     <sheet name="Selic_IPCA_2003_2016" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="DBGG_Fluxos_Conta_Unica" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="DBGG_Simulacao_Conta_Unica" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="Base_Monetaria_IPCA" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Macrometrica_Fluxos" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Macrometrica_DBGG" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="Base_Monetaria_IPCA" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10793,6 +10795,1266 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>pib_oficial</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>delta_pib</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>pib_cf</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>delta_pib_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>renuncia_estatica</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>receita_ciclo</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>renuncia_liquida</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bndes</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>fluxo_estatico</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fluxo_macrometrico</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>vazamento</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>selic_pct</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>dbgg</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>dbgg_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1717950.4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-9210.707852910051</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1708739.69214709</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.5361451560481636</v>
+      </c>
+      <c r="F2" t="n">
+        <v>13935.51963227513</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-2330.309086786243</v>
+      </c>
+      <c r="H2" t="n">
+        <v>11605.21054548889</v>
+      </c>
+      <c r="I2" t="n">
+        <v>14546</v>
+      </c>
+      <c r="J2" t="n">
+        <v>28481.51963227513</v>
+      </c>
+      <c r="K2" t="n">
+        <v>26151.21054548889</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2330.309086786241</v>
+      </c>
+      <c r="M2" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1957751.2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-11315.78590597498</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1946435.414094025</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.5779991812021354</v>
+      </c>
+      <c r="F3" t="n">
+        <v>15880.71476493745</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-2862.89383421167</v>
+      </c>
+      <c r="H3" t="n">
+        <v>13017.82093072577</v>
+      </c>
+      <c r="I3" t="n">
+        <v>19854</v>
+      </c>
+      <c r="J3" t="n">
+        <v>35734.71476493745</v>
+      </c>
+      <c r="K3" t="n">
+        <v>32871.82093072578</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2862.893834211667</v>
+      </c>
+      <c r="M3" t="n">
+        <v>16.24</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2170584.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-12295.11291694151</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2158289.387083059</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.5664424912709694</v>
+      </c>
+      <c r="F4" t="n">
+        <v>17607.15729235378</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-3110.663567986204</v>
+      </c>
+      <c r="H4" t="n">
+        <v>14496.49372436758</v>
+      </c>
+      <c r="I4" t="n">
+        <v>21009</v>
+      </c>
+      <c r="J4" t="n">
+        <v>38616.15729235378</v>
+      </c>
+      <c r="K4" t="n">
+        <v>35505.49372436758</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3110.663567986201</v>
+      </c>
+      <c r="M4" t="n">
+        <v>19.04</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2409449.9</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-14689.89567826976</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2394760.00432173</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.6096784032849057</v>
+      </c>
+      <c r="F5" t="n">
+        <v>20907.8641956744</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-3716.54360660225</v>
+      </c>
+      <c r="H5" t="n">
+        <v>17191.32058907215</v>
+      </c>
+      <c r="I5" t="n">
+        <v>25307</v>
+      </c>
+      <c r="J5" t="n">
+        <v>46214.8641956744</v>
+      </c>
+      <c r="K5" t="n">
+        <v>42498.32058907214</v>
+      </c>
+      <c r="L5" t="n">
+        <v>3716.543606602252</v>
+      </c>
+      <c r="M5" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1336644.9</v>
+      </c>
+      <c r="O5" t="n">
+        <v>55.48</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2720262.9</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-18135.10751613008</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2702127.79248387</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.6666674576244112</v>
+      </c>
+      <c r="F6" t="n">
+        <v>23604.92629032519</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-4588.18220158091</v>
+      </c>
+      <c r="H6" t="n">
+        <v>19016.74408874428</v>
+      </c>
+      <c r="I6" t="n">
+        <v>34772.548</v>
+      </c>
+      <c r="J6" t="n">
+        <v>58377.47429032519</v>
+      </c>
+      <c r="K6" t="n">
+        <v>53789.29208874428</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4588.182201580908</v>
+      </c>
+      <c r="M6" t="n">
+        <v>11.84</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1542851.83</v>
+      </c>
+      <c r="O6" t="n">
+        <v>56.72</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>3109803.1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-23464.16942056402</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3086338.930579436</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.7545226712444918</v>
+      </c>
+      <c r="F7" t="n">
+        <v>26985.13917641003</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-5936.434863402697</v>
+      </c>
+      <c r="H7" t="n">
+        <v>21048.70431300734</v>
+      </c>
+      <c r="I7" t="n">
+        <v>50680.455</v>
+      </c>
+      <c r="J7" t="n">
+        <v>77665.59417641003</v>
+      </c>
+      <c r="K7" t="n">
+        <v>71729.15931300735</v>
+      </c>
+      <c r="L7" t="n">
+        <v>5936.434863402683</v>
+      </c>
+      <c r="M7" t="n">
+        <v>12.48</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1740887.81</v>
+      </c>
+      <c r="O7" t="n">
+        <v>55.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3333039.4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-24857.88652907954</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3308181.51347092</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-0.7458023607245551</v>
+      </c>
+      <c r="F8" t="n">
+        <v>28922.25944769886</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-6289.045291857126</v>
+      </c>
+      <c r="H8" t="n">
+        <v>22633.21415584174</v>
+      </c>
+      <c r="I8" t="n">
+        <v>53155.931</v>
+      </c>
+      <c r="J8" t="n">
+        <v>82078.19044769886</v>
+      </c>
+      <c r="K8" t="n">
+        <v>75789.14515584173</v>
+      </c>
+      <c r="L8" t="n">
+        <v>6289.045291857125</v>
+      </c>
+      <c r="M8" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1973423.68</v>
+      </c>
+      <c r="O8" t="n">
+        <v>59.21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>3885847</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-40229.45910715045</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3845617.54089285</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-1.035281602882214</v>
+      </c>
+      <c r="F9" t="n">
+        <v>33719.21589287611</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-10178.05315410907</v>
+      </c>
+      <c r="H9" t="n">
+        <v>23541.16273876705</v>
+      </c>
+      <c r="I9" t="n">
+        <v>106967.091</v>
+      </c>
+      <c r="J9" t="n">
+        <v>140686.3068928761</v>
+      </c>
+      <c r="K9" t="n">
+        <v>130508.253738767</v>
+      </c>
+      <c r="L9" t="n">
+        <v>10178.05315410906</v>
+      </c>
+      <c r="M9" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2011521.66</v>
+      </c>
+      <c r="O9" t="n">
+        <v>51.77</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B10" t="n">
+        <v>4376382</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-32710.41091015679</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4343671.589089843</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-0.747430432493251</v>
+      </c>
+      <c r="F10" t="n">
+        <v>37975.80540039198</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-8275.73396026967</v>
+      </c>
+      <c r="H10" t="n">
+        <v>29700.0714401223</v>
+      </c>
+      <c r="I10" t="n">
+        <v>70080.355</v>
+      </c>
+      <c r="J10" t="n">
+        <v>108056.160400392</v>
+      </c>
+      <c r="K10" t="n">
+        <v>99780.4264401223</v>
+      </c>
+      <c r="L10" t="n">
+        <v>8275.733960269659</v>
+      </c>
+      <c r="M10" t="n">
+        <v>11.61</v>
+      </c>
+      <c r="N10" t="n">
+        <v>2243603.72</v>
+      </c>
+      <c r="O10" t="n">
+        <v>51.27</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B11" t="n">
+        <v>4814760</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-33890.15770510836</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4780869.842294891</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-0.703880519592012</v>
+      </c>
+      <c r="F11" t="n">
+        <v>41779.80551277089</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-8574.209899392417</v>
+      </c>
+      <c r="H11" t="n">
+        <v>33205.59561337847</v>
+      </c>
+      <c r="I11" t="n">
+        <v>68712.942</v>
+      </c>
+      <c r="J11" t="n">
+        <v>110492.7475127709</v>
+      </c>
+      <c r="K11" t="n">
+        <v>101918.5376133785</v>
+      </c>
+      <c r="L11" t="n">
+        <v>8574.209899392416</v>
+      </c>
+      <c r="M11" t="n">
+        <v>8.48</v>
+      </c>
+      <c r="N11" t="n">
+        <v>2583946.35</v>
+      </c>
+      <c r="O11" t="n">
+        <v>53.67</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B12" t="n">
+        <v>5331619</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-43332.21651204579</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5288286.783487954</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-0.8127403048125869</v>
+      </c>
+      <c r="F12" t="n">
+        <v>46264.82003011448</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-10963.05077754759</v>
+      </c>
+      <c r="H12" t="n">
+        <v>35301.7692525669</v>
+      </c>
+      <c r="I12" t="n">
+        <v>99305.15399999999</v>
+      </c>
+      <c r="J12" t="n">
+        <v>145569.9740301145</v>
+      </c>
+      <c r="K12" t="n">
+        <v>134606.9232525669</v>
+      </c>
+      <c r="L12" t="n">
+        <v>10963.05077754759</v>
+      </c>
+      <c r="M12" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="N12" t="n">
+        <v>2747996.71</v>
+      </c>
+      <c r="O12" t="n">
+        <v>51.54</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B13" t="n">
+        <v>5778953</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-41754.8946288408</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5737198.10537116</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-0.7225339024013658</v>
+      </c>
+      <c r="F13" t="n">
+        <v>50146.53532210201</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-10563.98834109673</v>
+      </c>
+      <c r="H13" t="n">
+        <v>39582.54698100527</v>
+      </c>
+      <c r="I13" t="n">
+        <v>86785.122</v>
+      </c>
+      <c r="J13" t="n">
+        <v>136931.657322102</v>
+      </c>
+      <c r="K13" t="n">
+        <v>126367.6689810053</v>
+      </c>
+      <c r="L13" t="n">
+        <v>10563.98834109672</v>
+      </c>
+      <c r="M13" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="N13" t="n">
+        <v>3252448.55</v>
+      </c>
+      <c r="O13" t="n">
+        <v>56.28</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B14" t="n">
+        <v>5995787</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-33714.274</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5962072.726</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-0.5622993945582123</v>
+      </c>
+      <c r="F14" t="n">
+        <v>52028.1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-8529.711322000003</v>
+      </c>
+      <c r="H14" t="n">
+        <v>43498.388678</v>
+      </c>
+      <c r="I14" t="n">
+        <v>51612.136</v>
+      </c>
+      <c r="J14" t="n">
+        <v>103640.236</v>
+      </c>
+      <c r="K14" t="n">
+        <v>95110.52467799999</v>
+      </c>
+      <c r="L14" t="n">
+        <v>8529.711322000017</v>
+      </c>
+      <c r="M14" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="N14" t="n">
+        <v>3927523.06</v>
+      </c>
+      <c r="O14" t="n">
+        <v>65.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fluxo_macrometrico</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>emissao_evitada</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>juros_evitados</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>acum_fluxo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>saldo_selic</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dbgg_oficial</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>dbgg_mm_estoque</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dbgg_mm_selic</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>dbgg_oficial_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dbgg_mm_estoque_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dbgg_mm_selic_pct</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>delta_oficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B2" t="n">
+        <v>26151.21054548889</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-26151.21054548889</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>26151.21054548889</v>
+      </c>
+      <c r="F2" t="n">
+        <v>26151.21054548889</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B3" t="n">
+        <v>32871.82093072578</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-32871.82093072578</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4246.956592587395</v>
+      </c>
+      <c r="E3" t="n">
+        <v>59023.03147621467</v>
+      </c>
+      <c r="F3" t="n">
+        <v>63269.98806880206</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B4" t="n">
+        <v>35505.49372436758</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-35505.49372436758</v>
+      </c>
+      <c r="D4" t="n">
+        <v>12046.60572829991</v>
+      </c>
+      <c r="E4" t="n">
+        <v>94528.52520058225</v>
+      </c>
+      <c r="F4" t="n">
+        <v>110822.0875214696</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B5" t="n">
+        <v>42498.32058907214</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-42498.32058907214</v>
+      </c>
+      <c r="D5" t="n">
+        <v>16711.97079823761</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137026.8457896544</v>
+      </c>
+      <c r="F5" t="n">
+        <v>170032.3789087793</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1336644.9</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1199618.054210345</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1166612.521091221</v>
+      </c>
+      <c r="J5" t="n">
+        <v>55.48</v>
+      </c>
+      <c r="K5" t="n">
+        <v>50.09345621462867</v>
+      </c>
+      <c r="L5" t="n">
+        <v>48.71521651380015</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B6" t="n">
+        <v>53789.29208874428</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-53789.29208874428</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20131.83366279947</v>
+      </c>
+      <c r="E6" t="n">
+        <v>190816.1378783987</v>
+      </c>
+      <c r="F6" t="n">
+        <v>243953.5046603231</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1542851.83</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1352035.692121601</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1298898.325339677</v>
+      </c>
+      <c r="J6" t="n">
+        <v>56.72</v>
+      </c>
+      <c r="K6" t="n">
+        <v>50.03596409771475</v>
+      </c>
+      <c r="L6" t="n">
+        <v>48.06946321904687</v>
+      </c>
+      <c r="M6" t="n">
+        <v>206206.9300000002</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B7" t="n">
+        <v>71729.15931300735</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-71729.15931300735</v>
+      </c>
+      <c r="D7" t="n">
+        <v>30445.39738160832</v>
+      </c>
+      <c r="E7" t="n">
+        <v>262545.297191406</v>
+      </c>
+      <c r="F7" t="n">
+        <v>346128.0613549388</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1740887.81</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1478342.512808594</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1394759.748645061</v>
+      </c>
+      <c r="J7" t="n">
+        <v>55.98</v>
+      </c>
+      <c r="K7" t="n">
+        <v>47.89955173623937</v>
+      </c>
+      <c r="L7" t="n">
+        <v>45.19139926032706</v>
+      </c>
+      <c r="M7" t="n">
+        <v>198035.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B8" t="n">
+        <v>75789.14515584173</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-75789.14515584173</v>
+      </c>
+      <c r="D8" t="n">
+        <v>34335.90368640993</v>
+      </c>
+      <c r="E8" t="n">
+        <v>338334.4423472477</v>
+      </c>
+      <c r="F8" t="n">
+        <v>456253.1101971904</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1973423.68</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1635089.237652752</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1517170.56980281</v>
+      </c>
+      <c r="J8" t="n">
+        <v>59.21</v>
+      </c>
+      <c r="K8" t="n">
+        <v>49.42562042000012</v>
+      </c>
+      <c r="L8" t="n">
+        <v>45.86116461944088</v>
+      </c>
+      <c r="M8" t="n">
+        <v>232535.8699999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B9" t="n">
+        <v>130508.253738767</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-130508.253738767</v>
+      </c>
+      <c r="D9" t="n">
+        <v>44621.55417728522</v>
+      </c>
+      <c r="E9" t="n">
+        <v>468842.6960860148</v>
+      </c>
+      <c r="F9" t="n">
+        <v>631382.9181132426</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2011521.66</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1542678.963913985</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1380138.741886757</v>
+      </c>
+      <c r="J9" t="n">
+        <v>51.77</v>
+      </c>
+      <c r="K9" t="n">
+        <v>40.11524670640587</v>
+      </c>
+      <c r="L9" t="n">
+        <v>35.88861157436696</v>
+      </c>
+      <c r="M9" t="n">
+        <v>38097.97999999998</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B10" t="n">
+        <v>99780.4264401223</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-99780.4264401223</v>
+      </c>
+      <c r="D10" t="n">
+        <v>73303.55679294746</v>
+      </c>
+      <c r="E10" t="n">
+        <v>568623.1225261372</v>
+      </c>
+      <c r="F10" t="n">
+        <v>804466.9013463125</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2243603.72</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1674980.597473863</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1439136.818653688</v>
+      </c>
+      <c r="J10" t="n">
+        <v>51.27</v>
+      </c>
+      <c r="K10" t="n">
+        <v>38.56140049079613</v>
+      </c>
+      <c r="L10" t="n">
+        <v>33.13180541246303</v>
+      </c>
+      <c r="M10" t="n">
+        <v>232082.0600000003</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B11" t="n">
+        <v>101918.5376133785</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-101918.5376133785</v>
+      </c>
+      <c r="D11" t="n">
+        <v>68218.7932341673</v>
+      </c>
+      <c r="E11" t="n">
+        <v>670541.6601395156</v>
+      </c>
+      <c r="F11" t="n">
+        <v>974604.2321938582</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2583946.35</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1913404.689860485</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1609342.117806142</v>
+      </c>
+      <c r="J11" t="n">
+        <v>53.67</v>
+      </c>
+      <c r="K11" t="n">
+        <v>40.02210377980131</v>
+      </c>
+      <c r="L11" t="n">
+        <v>33.66211946555802</v>
+      </c>
+      <c r="M11" t="n">
+        <v>340342.6299999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B12" t="n">
+        <v>134606.9232525669</v>
+      </c>
+      <c r="C12" t="n">
+        <v>-134606.9232525669</v>
+      </c>
+      <c r="D12" t="n">
+        <v>80015.00746311576</v>
+      </c>
+      <c r="E12" t="n">
+        <v>805148.5833920825</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1189226.162909541</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2747996.71</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1942848.126607917</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1558770.547090459</v>
+      </c>
+      <c r="J12" t="n">
+        <v>51.54</v>
+      </c>
+      <c r="K12" t="n">
+        <v>36.73870586357437</v>
+      </c>
+      <c r="L12" t="n">
+        <v>29.47590800025321</v>
+      </c>
+      <c r="M12" t="n">
+        <v>164050.3599999999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B13" t="n">
+        <v>126367.6689810053</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-126367.6689810053</v>
+      </c>
+      <c r="D13" t="n">
+        <v>129744.5743734309</v>
+      </c>
+      <c r="E13" t="n">
+        <v>931516.2523730878</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1445338.406263977</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3252448.55</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2320932.297626912</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1807110.143736023</v>
+      </c>
+      <c r="J13" t="n">
+        <v>56.28</v>
+      </c>
+      <c r="K13" t="n">
+        <v>40.45410764976126</v>
+      </c>
+      <c r="L13" t="n">
+        <v>31.49813045577436</v>
+      </c>
+      <c r="M13" t="n">
+        <v>504451.8399999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B14" t="n">
+        <v>95110.52467799999</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-95110.52467799999</v>
+      </c>
+      <c r="D14" t="n">
+        <v>192085.4741924825</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1026626.777051088</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1732534.40513446</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3927523.06</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2900896.282948912</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2194988.654865541</v>
+      </c>
+      <c r="J14" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>48.65583524834233</v>
+      </c>
+      <c r="L14" t="n">
+        <v>36.81586514859867</v>
+      </c>
+      <c r="M14" t="n">
+        <v>675074.5100000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>